<commit_message>
Updates on progress of viewport tuning
</commit_message>
<xml_diff>
--- a/ManpWinUI/Documentation/Architecture/PHASE5_STEP5.6_TEST_RESULTS.xlsx
+++ b/ManpWinUI/Documentation/Architecture/PHASE5_STEP5.6_TEST_RESULTS.xlsx
@@ -8,23 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\source\repos\ManpLab\ManpWinUI\Documentation\Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4B83AC3-246D-49E5-A53A-6632FC9F2309}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9C0AA9F-B103-41FA-A87F-EBCEE7775CD1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="30720" windowHeight="12270" tabRatio="490" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="30720" windowHeight="12270" tabRatio="373" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PHASE5_STEP5.6_TEST_RESULTS" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PHASE5_STEP5.6_TEST_RESULTS!$A$1:$E$136</definedName>
-    <definedName name="Data">PHASE5_STEP5.6_TEST_RESULTS!$A$1:$I$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PHASE5_STEP5.6_TEST_RESULTS!$A$1:$E$156</definedName>
+    <definedName name="Data">PHASE5_STEP5.6_TEST_RESULTS!$A$1:$I$156</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="194">
   <si>
     <t>Group Name</t>
   </si>
@@ -89,27 +89,12 @@
     <t>Historical Fractals</t>
   </si>
   <si>
-    <t>Biomorphs</t>
-  </si>
-  <si>
-    <t>ChipMap</t>
-  </si>
-  <si>
     <t>MartinMap</t>
   </si>
   <si>
     <t>Hybrid Fractals</t>
   </si>
   <si>
-    <t>BifurcationMandel</t>
-  </si>
-  <si>
-    <t>BurningMandel</t>
-  </si>
-  <si>
-    <t>CelticBurningHybrid</t>
-  </si>
-  <si>
     <t>IFS</t>
   </si>
   <si>
@@ -308,9 +293,6 @@
     <t>Pass</t>
   </si>
   <si>
-    <t>Fail</t>
-  </si>
-  <si>
     <t>Halvorsen Attractor</t>
   </si>
   <si>
@@ -428,9 +410,6 @@
     <t>Sprott B Attractor</t>
   </si>
   <si>
-    <t>black screen</t>
-  </si>
-  <si>
     <t>Tetrate</t>
   </si>
   <si>
@@ -536,7 +515,97 @@
     <t>z^z + c</t>
   </si>
   <si>
-    <t>, zoomed out nothing</t>
+    <t>Collatz Fractal</t>
+  </si>
+  <si>
+    <t>Chip Map</t>
+  </si>
+  <si>
+    <t>Duffing Map</t>
+  </si>
+  <si>
+    <t>Pickover Biomorphs</t>
+  </si>
+  <si>
+    <t>yet another Mandelbrot</t>
+  </si>
+  <si>
+    <t>Pickover Stalks</t>
+  </si>
+  <si>
+    <t>Quaternion Julia (2D slice)</t>
+  </si>
+  <si>
+    <t>Sinusoidal Fractal</t>
+  </si>
+  <si>
+    <t>Bifurcation-Mandel</t>
+  </si>
+  <si>
+    <t>Burning Mandelbrot Hybrid</t>
+  </si>
+  <si>
+    <t>Celtic-Burning Ship Hybrid</t>
+  </si>
+  <si>
+    <t>Collatz-Style Hybrid</t>
+  </si>
+  <si>
+    <t>Exponential-Mandelbrot Blend</t>
+  </si>
+  <si>
+    <t>Exponential-Mandelbrot Hybrid</t>
+  </si>
+  <si>
+    <t>Magnet-Mandelbrot Hybrid</t>
+  </si>
+  <si>
+    <t>Mandelbrot-Burning Ship Hybrid</t>
+  </si>
+  <si>
+    <t>Multi-Power Cycle</t>
+  </si>
+  <si>
+    <t>Mutant Mandelbrot (Power Evolution)</t>
+  </si>
+  <si>
+    <t>Newton-Mandelbrot Blend</t>
+  </si>
+  <si>
+    <t>Perturbed Newton</t>
+  </si>
+  <si>
+    <t>Sierpinski-Mandelbrot Cross</t>
+  </si>
+  <si>
+    <t>Sine-Mandelbrot Hybrid</t>
+  </si>
+  <si>
+    <t>Tricorn-Phoenix Hybrid</t>
+  </si>
+  <si>
+    <t>twin Mandelbrots</t>
+  </si>
+  <si>
+    <t>Burning Ship (Power 4)</t>
+  </si>
+  <si>
+    <t>green meteor</t>
+  </si>
+  <si>
+    <t>green earthworm</t>
+  </si>
+  <si>
+    <t>Mandelbrot-Lambda Mix</t>
+  </si>
+  <si>
+    <t>egg with holes</t>
+  </si>
+  <si>
+    <t>fields of squares</t>
+  </si>
+  <si>
+    <t>Trig-Mandelbrot Blend</t>
   </si>
 </sst>
 </file>
@@ -869,7 +938,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -1004,6 +1073,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1049,7 +1127,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1090,6 +1168,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1516,22 +1605,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I187"/>
+  <dimension ref="A1:I207"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5.796875" style="2" customWidth="1"/>
-    <col min="2" max="3" width="17.53125" customWidth="1"/>
+    <col min="2" max="2" width="17.53125" customWidth="1"/>
+    <col min="3" max="3" width="21.46484375" customWidth="1"/>
     <col min="4" max="4" width="7.796875" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5.6640625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="9.19921875" style="2" customWidth="1"/>
-    <col min="7" max="7" width="7.3984375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="7" style="2" customWidth="1"/>
+    <col min="7" max="7" width="6.33203125" style="2" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
     <col min="9" max="9" width="17.265625" customWidth="1"/>
+    <col min="10" max="10" width="3.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="20.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" s="10" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>0</v>
@@ -1543,19 +1634,19 @@
         <v>2</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
@@ -1566,10 +1657,10 @@
         <v>3</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F2" s="13"/>
       <c r="G2" s="13"/>
@@ -1585,10 +1676,10 @@
         <v>3</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F3" s="13"/>
       <c r="G3" s="13"/>
@@ -1597,17 +1688,17 @@
     </row>
     <row r="4" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="2">
-        <f t="shared" ref="A4:A85" si="0">A3+1</f>
+        <f t="shared" ref="A4:A67" si="0">A3+1</f>
         <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F4" s="13"/>
       <c r="G4" s="13"/>
@@ -1623,10 +1714,10 @@
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F5" s="13"/>
       <c r="G5" s="13"/>
@@ -1642,10 +1733,10 @@
         <v>3</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F6" s="13"/>
       <c r="G6" s="13"/>
@@ -1661,10 +1752,10 @@
         <v>3</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
@@ -1680,10 +1771,10 @@
         <v>3</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" s="14"/>
@@ -1700,10 +1791,10 @@
         <v>5</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F9" s="13"/>
       <c r="G9" s="13"/>
@@ -1719,10 +1810,10 @@
         <v>5</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F10" s="13"/>
       <c r="G10" s="13"/>
@@ -1738,10 +1829,10 @@
         <v>5</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
@@ -1757,10 +1848,10 @@
         <v>5</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F12" s="13"/>
       <c r="G12" s="13"/>
@@ -1776,10 +1867,10 @@
         <v>5</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
@@ -1795,10 +1886,10 @@
         <v>5</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="14"/>
@@ -1815,10 +1906,10 @@
         <v>6</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
@@ -1834,10 +1925,10 @@
         <v>6</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F16" s="13"/>
       <c r="G16" s="13"/>
@@ -1853,13 +1944,13 @@
         <v>6</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="F17" s="13"/>
       <c r="G17" s="13"/>
@@ -1875,10 +1966,10 @@
         <v>6</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E18" s="8"/>
       <c r="F18" s="13"/>
@@ -1895,13 +1986,13 @@
         <v>6</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="F19" s="13"/>
       <c r="G19" s="13"/>
@@ -1917,10 +2008,10 @@
         <v>6</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E20" s="6"/>
       <c r="F20" s="14"/>
@@ -1937,10 +2028,10 @@
         <v>7</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F21" s="13"/>
       <c r="G21" s="13"/>
@@ -1956,10 +2047,10 @@
         <v>7</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>119</v>
+        <v>187</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E22" s="6"/>
       <c r="F22" s="14"/>
@@ -1976,10 +2067,10 @@
         <v>8</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F23" s="13"/>
       <c r="G23" s="13"/>
@@ -1995,10 +2086,10 @@
         <v>8</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F24" s="13"/>
       <c r="G24" s="13"/>
@@ -2014,10 +2105,10 @@
         <v>8</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F25" s="13"/>
       <c r="G25" s="13"/>
@@ -2033,10 +2124,10 @@
         <v>8</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F26" s="13"/>
       <c r="G26" s="13"/>
@@ -2052,10 +2143,10 @@
         <v>8</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F27" s="13"/>
       <c r="G27" s="13"/>
@@ -2071,10 +2162,10 @@
         <v>8</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F28" s="13"/>
       <c r="G28" s="13"/>
@@ -2090,10 +2181,10 @@
         <v>8</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F29" s="13"/>
       <c r="G29" s="13"/>
@@ -2109,10 +2200,10 @@
         <v>8</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F30" s="13"/>
       <c r="G30" s="13"/>
@@ -2128,10 +2219,10 @@
         <v>8</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F31" s="13"/>
       <c r="G31" s="13"/>
@@ -2147,10 +2238,10 @@
         <v>8</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F32" s="13"/>
       <c r="G32" s="13"/>
@@ -2166,10 +2257,10 @@
         <v>8</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F33" s="13"/>
       <c r="G33" s="13"/>
@@ -2185,13 +2276,13 @@
         <v>8</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="F34" s="14"/>
       <c r="G34" s="14"/>
@@ -2210,7 +2301,7 @@
         <v>4</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F35" s="13">
         <v>0</v>
@@ -2237,7 +2328,7 @@
         <v>10</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F36" s="13">
         <v>0</v>
@@ -2264,7 +2355,7 @@
         <v>11</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F37" s="13"/>
       <c r="G37" s="13"/>
@@ -2280,10 +2371,10 @@
         <v>9</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E38" s="6"/>
       <c r="F38" s="14"/>
@@ -2300,18 +2391,26 @@
         <v>12</v>
       </c>
       <c r="C39" s="17" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="F39" s="15"/>
-      <c r="G39" s="15"/>
-      <c r="H39" s="16"/>
-      <c r="I39" s="16"/>
+        <v>186</v>
+      </c>
+      <c r="F39" s="15">
+        <v>1</v>
+      </c>
+      <c r="G39" s="15">
+        <v>0</v>
+      </c>
+      <c r="H39" s="16">
+        <v>6</v>
+      </c>
+      <c r="I39" s="16">
+        <v>3.375</v>
+      </c>
     </row>
     <row r="40" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A40" s="2">
@@ -2325,7 +2424,7 @@
         <v>13</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F40" s="13"/>
       <c r="G40" s="13"/>
@@ -2341,10 +2440,10 @@
         <v>12</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F41" s="13">
         <v>-1.5</v>
@@ -2360,7 +2459,7 @@
       </c>
     </row>
     <row r="42" spans="1:9" ht="20.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A42" s="5">
+      <c r="A42" s="2">
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
@@ -2368,10 +2467,10 @@
         <v>12</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E42" s="6"/>
       <c r="F42" s="14"/>
@@ -2388,10 +2487,10 @@
         <v>15</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F43" s="13"/>
       <c r="G43" s="13"/>
@@ -2407,10 +2506,10 @@
         <v>15</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F44" s="13"/>
       <c r="G44" s="13"/>
@@ -2426,10 +2525,10 @@
         <v>15</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F45" s="13"/>
       <c r="G45" s="13"/>
@@ -2438,17 +2537,17 @@
     </row>
     <row r="46" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A46" s="2">
-        <f t="shared" ref="A46:A49" si="1">A45+1</f>
+        <f t="shared" si="0"/>
         <v>45</v>
       </c>
       <c r="B46" t="s">
         <v>15</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F46" s="13"/>
       <c r="G46" s="13"/>
@@ -2457,17 +2556,17 @@
     </row>
     <row r="47" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A47" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>46</v>
       </c>
       <c r="B47" t="s">
         <v>15</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F47" s="13"/>
       <c r="G47" s="13"/>
@@ -2476,17 +2575,17 @@
     </row>
     <row r="48" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A48" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>47</v>
       </c>
       <c r="B48" t="s">
         <v>15</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F48" s="13"/>
       <c r="G48" s="13"/>
@@ -2494,18 +2593,18 @@
       <c r="I48" s="11"/>
     </row>
     <row r="49" spans="1:9" ht="20.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A49" s="5">
-        <f t="shared" si="1"/>
+      <c r="A49" s="2">
+        <f t="shared" si="0"/>
         <v>48</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>15</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E49" s="6"/>
       <c r="F49" s="14"/>
@@ -2515,17 +2614,17 @@
     </row>
     <row r="50" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A50" s="2">
-        <f>A45+1</f>
-        <v>45</v>
+        <f t="shared" si="0"/>
+        <v>49</v>
       </c>
       <c r="B50" t="s">
         <v>16</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F50" s="13"/>
       <c r="G50" s="13"/>
@@ -2535,16 +2634,16 @@
     <row r="51" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" s="2">
         <f t="shared" si="0"/>
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B51" t="s">
         <v>16</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F51" s="13"/>
       <c r="G51" s="13"/>
@@ -2554,16 +2653,16 @@
     <row r="52" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A52" s="2">
         <f t="shared" si="0"/>
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B52" t="s">
         <v>16</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F52" s="13"/>
       <c r="G52" s="13"/>
@@ -2571,18 +2670,18 @@
       <c r="I52" s="11"/>
     </row>
     <row r="53" spans="1:9" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A53" s="5">
-        <f t="shared" ref="A53" si="2">A52+1</f>
-        <v>48</v>
+      <c r="A53" s="2">
+        <f t="shared" si="0"/>
+        <v>52</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>16</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E53" s="6"/>
       <c r="F53" s="14"/>
@@ -2592,17 +2691,17 @@
     </row>
     <row r="54" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A54" s="2">
-        <f>A53+1</f>
-        <v>49</v>
+        <f t="shared" si="0"/>
+        <v>53</v>
       </c>
       <c r="B54" t="s">
         <v>17</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F54" s="13">
         <v>-0.5</v>
@@ -2619,17 +2718,17 @@
     </row>
     <row r="55" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A55" s="2">
-        <f>A54+1</f>
-        <v>50</v>
+        <f t="shared" si="0"/>
+        <v>54</v>
       </c>
       <c r="B55" t="s">
         <v>17</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F55" s="13">
         <v>-0.6</v>
@@ -2646,17 +2745,17 @@
     </row>
     <row r="56" spans="1:9" ht="27.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A56" s="2">
-        <f>A55+1</f>
-        <v>51</v>
+        <f t="shared" si="0"/>
+        <v>55</v>
       </c>
       <c r="B56" t="s">
         <v>17</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F56" s="13">
         <v>-0.4</v>
@@ -2673,17 +2772,17 @@
     </row>
     <row r="57" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A57" s="2">
-        <f>A56+1</f>
-        <v>52</v>
+        <f t="shared" si="0"/>
+        <v>56</v>
       </c>
       <c r="B57" t="s">
         <v>17</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F57" s="13">
         <v>-0.8</v>
@@ -2700,17 +2799,17 @@
     </row>
     <row r="58" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A58" s="2">
-        <f>A57+1</f>
-        <v>53</v>
+        <f t="shared" si="0"/>
+        <v>57</v>
       </c>
       <c r="B58" t="s">
         <v>17</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F58" s="13">
         <v>-0.5</v>
@@ -2727,20 +2826,20 @@
     </row>
     <row r="59" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A59" s="2">
-        <f>A58+1</f>
-        <v>54</v>
+        <f t="shared" si="0"/>
+        <v>58</v>
       </c>
       <c r="B59" t="s">
         <v>17</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="F59" s="13"/>
       <c r="G59" s="13"/>
@@ -2749,17 +2848,17 @@
     </row>
     <row r="60" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A60" s="2">
-        <f>A59+1</f>
-        <v>55</v>
+        <f t="shared" si="0"/>
+        <v>59</v>
       </c>
       <c r="B60" t="s">
         <v>17</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F60" s="13">
         <v>0</v>
@@ -2776,17 +2875,17 @@
     </row>
     <row r="61" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A61" s="2">
-        <f>A60+1</f>
-        <v>56</v>
+        <f t="shared" si="0"/>
+        <v>60</v>
       </c>
       <c r="B61" t="s">
         <v>18</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F61" s="13">
         <v>-0.5</v>
@@ -2803,32 +2902,32 @@
     </row>
     <row r="62" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A62" s="2">
-        <f t="shared" ref="A62:A78" si="3">A61+1</f>
-        <v>57</v>
+        <f t="shared" si="0"/>
+        <v>61</v>
       </c>
       <c r="B62" t="s">
         <v>18</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="63" spans="1:9" ht="20.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A63" s="5">
-        <f t="shared" si="3"/>
-        <v>58</v>
+      <c r="A63" s="2">
+        <f t="shared" si="0"/>
+        <v>62</v>
       </c>
       <c r="B63" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E63" s="6"/>
       <c r="F63" s="14">
@@ -2846,17 +2945,17 @@
     </row>
     <row r="64" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A64" s="2">
-        <f t="shared" si="3"/>
-        <v>59</v>
+        <f t="shared" si="0"/>
+        <v>63</v>
       </c>
       <c r="B64" t="s">
         <v>19</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F64" s="13">
         <v>0.5</v>
@@ -2873,17 +2972,17 @@
     </row>
     <row r="65" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A65" s="2">
-        <f t="shared" si="3"/>
-        <v>60</v>
+        <f t="shared" si="0"/>
+        <v>64</v>
       </c>
       <c r="B65" t="s">
         <v>19</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F65" s="13"/>
       <c r="G65" s="13"/>
@@ -2892,17 +2991,17 @@
     </row>
     <row r="66" spans="1:9" ht="31.9" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A66" s="2">
-        <f t="shared" si="3"/>
-        <v>61</v>
+        <f t="shared" si="0"/>
+        <v>65</v>
       </c>
       <c r="B66" t="s">
         <v>19</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F66" s="13">
         <v>-1</v>
@@ -2919,17 +3018,17 @@
     </row>
     <row r="67" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A67" s="2">
-        <f t="shared" si="3"/>
-        <v>62</v>
+        <f t="shared" si="0"/>
+        <v>66</v>
       </c>
       <c r="B67" t="s">
         <v>19</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F67" s="13"/>
       <c r="G67" s="13"/>
@@ -2938,17 +3037,17 @@
     </row>
     <row r="68" spans="1:9" ht="31.9" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A68" s="2">
-        <f t="shared" si="3"/>
-        <v>63</v>
+        <f t="shared" ref="A68:A131" si="1">A67+1</f>
+        <v>67</v>
       </c>
       <c r="B68" t="s">
         <v>19</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F68" s="13">
         <v>-2.5</v>
@@ -2965,17 +3064,17 @@
     </row>
     <row r="69" spans="1:9" ht="34.9" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A69" s="2">
-        <f t="shared" si="3"/>
-        <v>64</v>
+        <f t="shared" si="1"/>
+        <v>68</v>
       </c>
       <c r="B69" t="s">
         <v>19</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F69" s="13">
         <v>0</v>
@@ -2992,61 +3091,77 @@
     </row>
     <row r="70" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A70" s="2">
-        <f t="shared" si="3"/>
-        <v>65</v>
+        <f t="shared" si="1"/>
+        <v>69</v>
       </c>
       <c r="B70" t="s">
         <v>19</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="F70" s="13"/>
-      <c r="G70" s="13"/>
-      <c r="H70" s="11"/>
-      <c r="I70" s="11"/>
+        <v>188</v>
+      </c>
+      <c r="F70" s="13">
+        <v>0.875</v>
+      </c>
+      <c r="G70" s="13">
+        <v>0</v>
+      </c>
+      <c r="H70" s="11">
+        <v>0.375</v>
+      </c>
+      <c r="I70" s="11">
+        <v>0.2109375</v>
+      </c>
     </row>
     <row r="71" spans="1:9" ht="34.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A71" s="2">
-        <f t="shared" si="3"/>
-        <v>66</v>
+        <f t="shared" si="1"/>
+        <v>70</v>
       </c>
       <c r="B71" t="s">
         <v>19</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="F71" s="13"/>
-      <c r="G71" s="13"/>
-      <c r="H71" s="11"/>
-      <c r="I71" s="11"/>
+        <v>189</v>
+      </c>
+      <c r="F71" s="13">
+        <v>0.24</v>
+      </c>
+      <c r="G71" s="13">
+        <v>-0.3</v>
+      </c>
+      <c r="H71" s="11">
+        <v>1.9350213897999999</v>
+      </c>
+      <c r="I71" s="11">
+        <v>1.0884495317</v>
+      </c>
     </row>
     <row r="72" spans="1:9" ht="31.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A72" s="2">
-        <f t="shared" si="3"/>
-        <v>67</v>
+        <f t="shared" si="1"/>
+        <v>71</v>
       </c>
       <c r="B72" t="s">
         <v>19</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F72" s="13">
         <v>-1.75</v>
@@ -3063,17 +3178,17 @@
     </row>
     <row r="73" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A73" s="2">
-        <f t="shared" si="3"/>
-        <v>68</v>
+        <f t="shared" si="1"/>
+        <v>72</v>
       </c>
       <c r="B73" t="s">
         <v>19</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F73" s="13">
         <v>0.75</v>
@@ -3089,18 +3204,18 @@
       </c>
     </row>
     <row r="74" spans="1:9" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A74" s="5">
-        <f t="shared" si="3"/>
-        <v>69</v>
+      <c r="A74" s="2">
+        <f t="shared" si="1"/>
+        <v>73</v>
       </c>
       <c r="B74" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E74" s="6"/>
       <c r="F74" s="14">
@@ -3118,14 +3233,17 @@
     </row>
     <row r="75" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A75" s="2">
-        <f t="shared" si="3"/>
-        <v>70</v>
+        <f t="shared" si="1"/>
+        <v>74</v>
       </c>
       <c r="B75" t="s">
         <v>20</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>21</v>
+        <v>164</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>88</v>
       </c>
       <c r="F75" s="13"/>
       <c r="G75" s="13"/>
@@ -3134,14 +3252,17 @@
     </row>
     <row r="76" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A76" s="2">
-        <f t="shared" si="3"/>
-        <v>71</v>
+        <f t="shared" si="1"/>
+        <v>75</v>
       </c>
       <c r="B76" t="s">
         <v>20</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>22</v>
+        <v>163</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>88</v>
       </c>
       <c r="F76" s="13"/>
       <c r="G76" s="13"/>
@@ -3150,46 +3271,74 @@
     </row>
     <row r="77" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A77" s="2">
-        <f t="shared" si="3"/>
-        <v>72</v>
+        <f t="shared" si="1"/>
+        <v>76</v>
       </c>
       <c r="B77" t="s">
         <v>20</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F77" s="13"/>
-      <c r="G77" s="13"/>
-      <c r="H77" s="11"/>
-      <c r="I77" s="11"/>
+        <v>165</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F77" s="13">
+        <v>0</v>
+      </c>
+      <c r="G77" s="13">
+        <v>0</v>
+      </c>
+      <c r="H77" s="11">
+        <v>6.7677102075000004</v>
+      </c>
+      <c r="I77" s="11">
+        <v>3.8068369917</v>
+      </c>
     </row>
     <row r="78" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A78" s="2">
-        <f t="shared" si="3"/>
-        <v>73</v>
+        <f t="shared" si="1"/>
+        <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F78" s="13"/>
-      <c r="G78" s="13"/>
-      <c r="H78" s="11"/>
-      <c r="I78" s="11"/>
+        <v>21</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F78" s="13">
+        <v>0</v>
+      </c>
+      <c r="G78" s="13">
+        <v>0</v>
+      </c>
+      <c r="H78" s="11">
+        <v>442.66476249999999</v>
+      </c>
+      <c r="I78" s="11">
+        <v>248.99892890999999</v>
+      </c>
     </row>
     <row r="79" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A79" s="2">
-        <f t="shared" si="0"/>
-        <v>74</v>
+        <f t="shared" si="1"/>
+        <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>26</v>
+        <v>166</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>167</v>
       </c>
       <c r="F79" s="13"/>
       <c r="G79" s="13"/>
@@ -3198,350 +3347,565 @@
     </row>
     <row r="80" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A80" s="2">
-        <f t="shared" si="0"/>
-        <v>75</v>
+        <f t="shared" si="1"/>
+        <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F80" s="13"/>
-      <c r="G80" s="13"/>
-      <c r="H80" s="11"/>
-      <c r="I80" s="11"/>
-    </row>
-    <row r="81" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+        <v>168</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F80" s="13">
+        <v>-0.75</v>
+      </c>
+      <c r="G80" s="13">
+        <v>0</v>
+      </c>
+      <c r="H80" s="11">
+        <v>3.9272543837999998</v>
+      </c>
+      <c r="I80" s="11">
+        <v>2.2090805910000002</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A81" s="2">
-        <f t="shared" si="0"/>
-        <v>76</v>
+        <f t="shared" si="1"/>
+        <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>29</v>
+        <v>169</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>88</v>
       </c>
       <c r="F81" s="13"/>
       <c r="G81" s="13"/>
       <c r="H81" s="11"/>
       <c r="I81" s="11"/>
     </row>
-    <row r="82" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:9" ht="20.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A82" s="2">
-        <f t="shared" si="0"/>
-        <v>77</v>
-      </c>
-      <c r="B82" t="s">
-        <v>28</v>
-      </c>
-      <c r="C82" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F82" s="13"/>
-      <c r="G82" s="13"/>
-      <c r="H82" s="11"/>
-      <c r="I82" s="11"/>
-    </row>
-    <row r="83" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+        <f t="shared" si="1"/>
+        <v>81</v>
+      </c>
+      <c r="B82" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="C82" s="19" t="s">
+        <v>170</v>
+      </c>
+      <c r="D82" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="E82" s="19"/>
+      <c r="F82" s="21"/>
+      <c r="G82" s="21"/>
+      <c r="H82" s="22"/>
+      <c r="I82" s="22"/>
+    </row>
+    <row r="83" spans="1:9" ht="20.350000000000001" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
       <c r="A83" s="2">
-        <f t="shared" si="0"/>
-        <v>78</v>
+        <f t="shared" si="1"/>
+        <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F83" s="13"/>
-      <c r="G83" s="13"/>
-      <c r="H83" s="11"/>
-      <c r="I83" s="11"/>
-    </row>
-    <row r="84" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+        <v>171</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F83" s="13">
+        <v>1</v>
+      </c>
+      <c r="G83" s="13">
+        <v>0</v>
+      </c>
+      <c r="H83" s="11">
+        <v>6.6504798242999996</v>
+      </c>
+      <c r="I83" s="11">
+        <v>3.7408990110000002</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A84" s="2">
-        <f t="shared" si="0"/>
-        <v>79</v>
+        <f t="shared" si="1"/>
+        <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F84" s="13"/>
-      <c r="G84" s="13"/>
-      <c r="H84" s="11"/>
-      <c r="I84" s="11"/>
+        <v>172</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F84" s="13">
+        <v>-0.5</v>
+      </c>
+      <c r="G84" s="13">
+        <v>0</v>
+      </c>
+      <c r="H84" s="11">
+        <v>3.7942978950000001</v>
+      </c>
+      <c r="I84" s="11">
+        <v>2.1342925659</v>
+      </c>
     </row>
     <row r="85" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A85" s="2">
-        <f t="shared" si="0"/>
-        <v>80</v>
+        <f t="shared" si="1"/>
+        <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F85" s="13"/>
-      <c r="G85" s="13"/>
-      <c r="H85" s="11"/>
-      <c r="I85" s="11"/>
+        <v>141</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F85" s="13">
+        <v>-0.75</v>
+      </c>
+      <c r="G85" s="13">
+        <v>0</v>
+      </c>
+      <c r="H85" s="11">
+        <v>4.2857142857000001</v>
+      </c>
+      <c r="I85" s="11">
+        <v>2.4107142857000001</v>
+      </c>
     </row>
     <row r="86" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A86" s="2">
-        <f t="shared" ref="A86:A137" si="4">A85+1</f>
-        <v>81</v>
+        <f t="shared" si="1"/>
+        <v>85</v>
       </c>
       <c r="B86" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="F86" s="13"/>
-      <c r="G86" s="13"/>
-      <c r="H86" s="11"/>
-      <c r="I86" s="11"/>
+        <v>173</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F86" s="13">
+        <v>-0.5</v>
+      </c>
+      <c r="G86" s="13">
+        <v>0</v>
+      </c>
+      <c r="H86" s="11">
+        <v>4.1877356094999998</v>
+      </c>
+      <c r="I86" s="11">
+        <v>2.3556012803000002</v>
+      </c>
     </row>
     <row r="87" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A87" s="2">
-        <f t="shared" si="4"/>
-        <v>82</v>
+        <f t="shared" si="1"/>
+        <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F87" s="13"/>
-      <c r="G87" s="13"/>
-      <c r="H87" s="11"/>
-      <c r="I87" s="11"/>
-    </row>
-    <row r="88" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+        <v>174</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F87" s="13">
+        <v>0</v>
+      </c>
+      <c r="G87" s="13">
+        <v>0</v>
+      </c>
+      <c r="H87" s="11">
+        <v>6</v>
+      </c>
+      <c r="I87" s="11">
+        <v>3.375</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" ht="35.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A88" s="2">
-        <f t="shared" si="4"/>
-        <v>83</v>
+        <f t="shared" si="1"/>
+        <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F88" s="13"/>
-      <c r="G88" s="13"/>
-      <c r="H88" s="11"/>
-      <c r="I88" s="11"/>
-    </row>
-    <row r="89" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+        <v>175</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F88" s="13">
+        <v>-1.4</v>
+      </c>
+      <c r="G88" s="13">
+        <v>0</v>
+      </c>
+      <c r="H88" s="11">
+        <v>3</v>
+      </c>
+      <c r="I88" s="11">
+        <v>1.6875</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A89" s="2">
-        <f t="shared" si="4"/>
-        <v>84</v>
+        <f t="shared" si="1"/>
+        <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F89" s="13"/>
-      <c r="G89" s="13"/>
-      <c r="H89" s="11"/>
-      <c r="I89" s="11"/>
-    </row>
-    <row r="90" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+        <v>176</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F89" s="13">
+        <v>-1.4</v>
+      </c>
+      <c r="G89" s="13">
+        <v>0</v>
+      </c>
+      <c r="H89" s="11">
+        <v>5.6960146865999999</v>
+      </c>
+      <c r="I89" s="11">
+        <v>3.2040082611999998</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A90" s="2">
-        <f t="shared" si="4"/>
-        <v>85</v>
+        <f t="shared" si="1"/>
+        <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F90" s="13"/>
-      <c r="G90" s="13"/>
-      <c r="H90" s="11"/>
-      <c r="I90" s="11"/>
-    </row>
-    <row r="91" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+        <v>177</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F90" s="13">
+        <v>-2</v>
+      </c>
+      <c r="G90" s="13">
+        <v>0</v>
+      </c>
+      <c r="H90" s="11">
+        <v>19.878954426</v>
+      </c>
+      <c r="I90" s="11">
+        <v>11.181911864</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A91" s="2">
-        <f t="shared" si="4"/>
-        <v>86</v>
+        <f t="shared" si="1"/>
+        <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F91" s="13"/>
-      <c r="G91" s="13"/>
-      <c r="H91" s="11"/>
-      <c r="I91" s="11"/>
-    </row>
-    <row r="92" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+        <v>178</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F91" s="13">
+        <v>0</v>
+      </c>
+      <c r="G91" s="13">
+        <v>0</v>
+      </c>
+      <c r="H91" s="11">
+        <v>4.5202694987000003</v>
+      </c>
+      <c r="I91" s="11">
+        <v>2.542651593</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A92" s="2">
-        <f t="shared" si="4"/>
-        <v>87</v>
+        <f t="shared" si="1"/>
+        <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="F92" s="13"/>
-      <c r="G92" s="13"/>
-      <c r="H92" s="11"/>
-      <c r="I92" s="11"/>
-    </row>
-    <row r="93" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+        <v>190</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F92" s="13">
+        <v>-0.75</v>
+      </c>
+      <c r="G92" s="13">
+        <v>0</v>
+      </c>
+      <c r="H92" s="11">
+        <v>8.31700354</v>
+      </c>
+      <c r="I92" s="11">
+        <v>4.6783144913000001</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A93" s="2">
-        <f t="shared" si="4"/>
-        <v>88</v>
+        <f t="shared" si="1"/>
+        <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>45</v>
+        <v>179</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>88</v>
       </c>
       <c r="F93" s="13"/>
       <c r="G93" s="13"/>
       <c r="H93" s="11"/>
       <c r="I93" s="11"/>
     </row>
-    <row r="94" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A94" s="2">
-        <f t="shared" si="4"/>
-        <v>89</v>
+        <f t="shared" si="1"/>
+        <v>93</v>
       </c>
       <c r="B94" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F94" s="13"/>
-      <c r="G94" s="13"/>
-      <c r="H94" s="11"/>
-      <c r="I94" s="11"/>
-    </row>
-    <row r="95" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+        <v>180</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F94" s="13">
+        <v>-0.5</v>
+      </c>
+      <c r="G94" s="13">
+        <v>0</v>
+      </c>
+      <c r="H94" s="11">
+        <v>3</v>
+      </c>
+      <c r="I94" s="11">
+        <v>1.6875</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A95" s="2">
-        <f t="shared" si="4"/>
-        <v>90</v>
+        <f t="shared" si="1"/>
+        <v>94</v>
       </c>
       <c r="B95" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F95" s="13"/>
-      <c r="G95" s="13"/>
-      <c r="H95" s="11"/>
-      <c r="I95" s="11"/>
-    </row>
-    <row r="96" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+        <v>181</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E95" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="F95" s="13">
+        <v>-0.75</v>
+      </c>
+      <c r="G95" s="13">
+        <v>0</v>
+      </c>
+      <c r="H95" s="11">
+        <v>10.867649183999999</v>
+      </c>
+      <c r="I95" s="11">
+        <v>6.1130526660999998</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A96" s="2">
-        <f t="shared" si="4"/>
-        <v>91</v>
+        <f t="shared" si="1"/>
+        <v>95</v>
       </c>
       <c r="B96" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="F96" s="13"/>
-      <c r="G96" s="13"/>
-      <c r="H96" s="11"/>
-      <c r="I96" s="11"/>
-    </row>
-    <row r="97" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+        <v>182</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F96" s="13">
+        <v>0</v>
+      </c>
+      <c r="G96" s="13">
+        <v>0</v>
+      </c>
+      <c r="H96" s="11">
+        <v>20</v>
+      </c>
+      <c r="I96" s="11">
+        <v>11.25</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" ht="57" x14ac:dyDescent="0.45">
       <c r="A97" s="2">
-        <f t="shared" si="4"/>
-        <v>92</v>
+        <f t="shared" si="1"/>
+        <v>96</v>
       </c>
       <c r="B97" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F97" s="13"/>
-      <c r="G97" s="13"/>
-      <c r="H97" s="11"/>
-      <c r="I97" s="11"/>
-    </row>
-    <row r="98" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+        <v>183</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E97" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="F97" s="13">
+        <v>0</v>
+      </c>
+      <c r="G97" s="13">
+        <v>0</v>
+      </c>
+      <c r="H97" s="11">
+        <v>7.5</v>
+      </c>
+      <c r="I97" s="11">
+        <v>4.21875</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A98" s="2">
-        <f t="shared" si="4"/>
-        <v>93</v>
+        <f t="shared" si="1"/>
+        <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F98" s="13"/>
-      <c r="G98" s="13"/>
-      <c r="H98" s="11"/>
-      <c r="I98" s="11"/>
-    </row>
-    <row r="99" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+        <v>184</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F98" s="13">
+        <v>0</v>
+      </c>
+      <c r="G98" s="13">
+        <v>0</v>
+      </c>
+      <c r="H98" s="11">
+        <v>4</v>
+      </c>
+      <c r="I98" s="11">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A99" s="2">
-        <f t="shared" si="4"/>
-        <v>94</v>
+        <f t="shared" si="1"/>
+        <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F99" s="13"/>
-      <c r="G99" s="13"/>
-      <c r="H99" s="11"/>
-      <c r="I99" s="11"/>
-    </row>
-    <row r="100" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+        <v>185</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F99" s="13">
+        <v>-0.58126820893451703</v>
+      </c>
+      <c r="G99" s="13">
+        <v>-0.109703194367369</v>
+      </c>
+      <c r="H99" s="11">
+        <v>1.8124306325999999</v>
+      </c>
+      <c r="I99" s="11">
+        <v>1.0194922309000001</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" ht="28.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A100" s="2">
-        <f t="shared" si="4"/>
-        <v>95</v>
-      </c>
-      <c r="B100" t="s">
-        <v>52</v>
-      </c>
-      <c r="C100" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F100" s="13"/>
-      <c r="G100" s="13"/>
-      <c r="H100" s="11"/>
-      <c r="I100" s="11"/>
+        <f t="shared" si="1"/>
+        <v>99</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C100" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="D100" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="E100" s="6"/>
+      <c r="F100" s="14">
+        <v>-0.36983592449361802</v>
+      </c>
+      <c r="G100" s="14">
+        <v>-1.44284128745837E-2</v>
+      </c>
+      <c r="H100" s="12">
+        <v>4.1593292608999999</v>
+      </c>
+      <c r="I100" s="12">
+        <v>2.3396227092999999</v>
+      </c>
     </row>
     <row r="101" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A101" s="2">
-        <f t="shared" si="4"/>
-        <v>96</v>
+        <f t="shared" si="1"/>
+        <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="F101" s="13"/>
       <c r="G101" s="13"/>
@@ -3550,14 +3914,14 @@
     </row>
     <row r="102" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A102" s="2">
-        <f t="shared" si="4"/>
-        <v>97</v>
+        <f t="shared" si="1"/>
+        <v>101</v>
       </c>
       <c r="B102" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="F102" s="13"/>
       <c r="G102" s="13"/>
@@ -3566,14 +3930,14 @@
     </row>
     <row r="103" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A103" s="2">
-        <f t="shared" si="4"/>
-        <v>98</v>
+        <f t="shared" si="1"/>
+        <v>102</v>
       </c>
       <c r="B103" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="F103" s="13"/>
       <c r="G103" s="13"/>
@@ -3582,14 +3946,14 @@
     </row>
     <row r="104" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A104" s="2">
-        <f t="shared" si="4"/>
-        <v>99</v>
+        <f t="shared" si="1"/>
+        <v>103</v>
       </c>
       <c r="B104" t="s">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="F104" s="13"/>
       <c r="G104" s="13"/>
@@ -3598,14 +3962,14 @@
     </row>
     <row r="105" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A105" s="2">
-        <f t="shared" si="4"/>
-        <v>100</v>
+        <f t="shared" si="1"/>
+        <v>104</v>
       </c>
       <c r="B105" t="s">
-        <v>60</v>
+        <v>27</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>57</v>
+        <v>29</v>
       </c>
       <c r="F105" s="13"/>
       <c r="G105" s="13"/>
@@ -3614,14 +3978,14 @@
     </row>
     <row r="106" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A106" s="2">
-        <f t="shared" si="4"/>
-        <v>101</v>
+        <f t="shared" si="1"/>
+        <v>105</v>
       </c>
       <c r="B106" t="s">
-        <v>60</v>
+        <v>27</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="F106" s="13"/>
       <c r="G106" s="13"/>
@@ -3630,14 +3994,14 @@
     </row>
     <row r="107" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A107" s="2">
-        <f t="shared" si="4"/>
-        <v>102</v>
+        <f t="shared" si="1"/>
+        <v>106</v>
       </c>
       <c r="B107" t="s">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="F107" s="13"/>
       <c r="G107" s="13"/>
@@ -3646,14 +4010,14 @@
     </row>
     <row r="108" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A108" s="2">
-        <f t="shared" si="4"/>
-        <v>103</v>
+        <f t="shared" si="1"/>
+        <v>107</v>
       </c>
       <c r="B108" t="s">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="F108" s="13"/>
       <c r="G108" s="13"/>
@@ -3662,14 +4026,14 @@
     </row>
     <row r="109" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A109" s="2">
-        <f t="shared" si="4"/>
-        <v>104</v>
+        <f t="shared" si="1"/>
+        <v>108</v>
       </c>
       <c r="B109" t="s">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="F109" s="13"/>
       <c r="G109" s="13"/>
@@ -3678,14 +4042,14 @@
     </row>
     <row r="110" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A110" s="2">
-        <f t="shared" si="4"/>
-        <v>105</v>
+        <f t="shared" si="1"/>
+        <v>109</v>
       </c>
       <c r="B110" t="s">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="F110" s="13"/>
       <c r="G110" s="13"/>
@@ -3694,14 +4058,14 @@
     </row>
     <row r="111" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A111" s="2">
-        <f t="shared" si="4"/>
-        <v>106</v>
+        <f t="shared" si="1"/>
+        <v>110</v>
       </c>
       <c r="B111" t="s">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>66</v>
+        <v>37</v>
       </c>
       <c r="F111" s="13"/>
       <c r="G111" s="13"/>
@@ -3710,14 +4074,14 @@
     </row>
     <row r="112" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A112" s="2">
-        <f t="shared" si="4"/>
-        <v>107</v>
+        <f t="shared" si="1"/>
+        <v>111</v>
       </c>
       <c r="B112" t="s">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="F112" s="13"/>
       <c r="G112" s="13"/>
@@ -3726,14 +4090,14 @@
     </row>
     <row r="113" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A113" s="2">
-        <f t="shared" si="4"/>
-        <v>108</v>
+        <f t="shared" si="1"/>
+        <v>112</v>
       </c>
       <c r="B113" t="s">
-        <v>65</v>
+        <v>39</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="F113" s="13"/>
       <c r="G113" s="13"/>
@@ -3742,14 +4106,14 @@
     </row>
     <row r="114" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A114" s="2">
-        <f t="shared" si="4"/>
-        <v>109</v>
+        <f t="shared" si="1"/>
+        <v>113</v>
       </c>
       <c r="B114" t="s">
-        <v>69</v>
+        <v>39</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="F114" s="13"/>
       <c r="G114" s="13"/>
@@ -3758,14 +4122,14 @@
     </row>
     <row r="115" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A115" s="2">
-        <f t="shared" si="4"/>
-        <v>110</v>
+        <f t="shared" si="1"/>
+        <v>114</v>
       </c>
       <c r="B115" t="s">
-        <v>69</v>
+        <v>39</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="F115" s="13"/>
       <c r="G115" s="13"/>
@@ -3774,14 +4138,14 @@
     </row>
     <row r="116" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A116" s="2">
-        <f t="shared" si="4"/>
-        <v>111</v>
+        <f t="shared" si="1"/>
+        <v>115</v>
       </c>
       <c r="B116" t="s">
-        <v>69</v>
+        <v>43</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="F116" s="13"/>
       <c r="G116" s="13"/>
@@ -3790,14 +4154,14 @@
     </row>
     <row r="117" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A117" s="2">
-        <f t="shared" si="4"/>
-        <v>112</v>
+        <f t="shared" si="1"/>
+        <v>116</v>
       </c>
       <c r="B117" t="s">
-        <v>73</v>
+        <v>43</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="F117" s="13"/>
       <c r="G117" s="13"/>
@@ -3806,14 +4170,14 @@
     </row>
     <row r="118" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A118" s="2">
-        <f t="shared" si="4"/>
-        <v>113</v>
+        <f t="shared" si="1"/>
+        <v>117</v>
       </c>
       <c r="B118" t="s">
-        <v>73</v>
+        <v>43</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>71</v>
+        <v>46</v>
       </c>
       <c r="F118" s="13"/>
       <c r="G118" s="13"/>
@@ -3822,14 +4186,14 @@
     </row>
     <row r="119" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A119" s="2">
-        <f t="shared" si="4"/>
-        <v>114</v>
+        <f t="shared" si="1"/>
+        <v>118</v>
       </c>
       <c r="B119" t="s">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="F119" s="13"/>
       <c r="G119" s="13"/>
@@ -3838,14 +4202,14 @@
     </row>
     <row r="120" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A120" s="2">
-        <f t="shared" si="4"/>
-        <v>115</v>
+        <f t="shared" si="1"/>
+        <v>119</v>
       </c>
       <c r="B120" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>75</v>
+        <v>49</v>
       </c>
       <c r="F120" s="13"/>
       <c r="G120" s="13"/>
@@ -3854,14 +4218,14 @@
     </row>
     <row r="121" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A121" s="2">
-        <f t="shared" si="4"/>
-        <v>116</v>
+        <f t="shared" si="1"/>
+        <v>120</v>
       </c>
       <c r="B121" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="F121" s="13"/>
       <c r="G121" s="13"/>
@@ -3870,14 +4234,14 @@
     </row>
     <row r="122" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A122" s="2">
-        <f t="shared" si="4"/>
-        <v>117</v>
+        <f t="shared" si="1"/>
+        <v>121</v>
       </c>
       <c r="B122" t="s">
-        <v>74</v>
+        <v>51</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>77</v>
+        <v>52</v>
       </c>
       <c r="F122" s="13"/>
       <c r="G122" s="13"/>
@@ -3886,14 +4250,14 @@
     </row>
     <row r="123" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A123" s="2">
-        <f t="shared" si="4"/>
-        <v>118</v>
+        <f t="shared" si="1"/>
+        <v>122</v>
       </c>
       <c r="B123" t="s">
-        <v>78</v>
+        <v>51</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>79</v>
+        <v>53</v>
       </c>
       <c r="F123" s="13"/>
       <c r="G123" s="13"/>
@@ -3902,14 +4266,14 @@
     </row>
     <row r="124" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A124" s="2">
-        <f t="shared" si="4"/>
-        <v>119</v>
+        <f t="shared" si="1"/>
+        <v>123</v>
       </c>
       <c r="B124" t="s">
-        <v>78</v>
+        <v>51</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>80</v>
+        <v>54</v>
       </c>
       <c r="F124" s="13"/>
       <c r="G124" s="13"/>
@@ -3918,14 +4282,14 @@
     </row>
     <row r="125" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A125" s="2">
-        <f t="shared" si="4"/>
-        <v>120</v>
+        <f t="shared" si="1"/>
+        <v>124</v>
       </c>
       <c r="B125" t="s">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>81</v>
+        <v>52</v>
       </c>
       <c r="F125" s="13"/>
       <c r="G125" s="13"/>
@@ -3934,14 +4298,14 @@
     </row>
     <row r="126" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A126" s="2">
-        <f t="shared" si="4"/>
-        <v>121</v>
+        <f t="shared" si="1"/>
+        <v>125</v>
       </c>
       <c r="B126" t="s">
-        <v>82</v>
+        <v>55</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>79</v>
+        <v>53</v>
       </c>
       <c r="F126" s="13"/>
       <c r="G126" s="13"/>
@@ -3950,14 +4314,14 @@
     </row>
     <row r="127" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A127" s="2">
-        <f t="shared" si="4"/>
-        <v>122</v>
+        <f t="shared" si="1"/>
+        <v>126</v>
       </c>
       <c r="B127" t="s">
-        <v>82</v>
+        <v>55</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>80</v>
+        <v>54</v>
       </c>
       <c r="F127" s="13"/>
       <c r="G127" s="13"/>
@@ -3966,14 +4330,14 @@
     </row>
     <row r="128" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A128" s="2">
-        <f t="shared" si="4"/>
-        <v>123</v>
+        <f t="shared" si="1"/>
+        <v>127</v>
       </c>
       <c r="B128" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="F128" s="13"/>
       <c r="G128" s="13"/>
@@ -3982,14 +4346,14 @@
     </row>
     <row r="129" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A129" s="2">
-        <f t="shared" si="4"/>
-        <v>124</v>
+        <f t="shared" si="1"/>
+        <v>128</v>
       </c>
       <c r="B129" t="s">
-        <v>83</v>
+        <v>56</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="F129" s="13"/>
       <c r="G129" s="13"/>
@@ -3998,14 +4362,14 @@
     </row>
     <row r="130" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A130" s="2">
-        <f t="shared" si="4"/>
-        <v>125</v>
+        <f t="shared" si="1"/>
+        <v>129</v>
       </c>
       <c r="B130" t="s">
-        <v>83</v>
+        <v>56</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>84</v>
+        <v>59</v>
       </c>
       <c r="F130" s="13"/>
       <c r="G130" s="13"/>
@@ -4014,14 +4378,14 @@
     </row>
     <row r="131" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A131" s="2">
-        <f t="shared" si="4"/>
-        <v>126</v>
+        <f t="shared" si="1"/>
+        <v>130</v>
       </c>
       <c r="B131" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>85</v>
+        <v>61</v>
       </c>
       <c r="F131" s="13"/>
       <c r="G131" s="13"/>
@@ -4030,14 +4394,14 @@
     </row>
     <row r="132" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A132" s="2">
-        <f t="shared" si="4"/>
-        <v>127</v>
+        <f t="shared" ref="A132:A156" si="2">A131+1</f>
+        <v>131</v>
       </c>
       <c r="B132" t="s">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="F132" s="13"/>
       <c r="G132" s="13"/>
@@ -4046,14 +4410,14 @@
     </row>
     <row r="133" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A133" s="2">
-        <f t="shared" si="4"/>
-        <v>128</v>
+        <f t="shared" si="2"/>
+        <v>132</v>
       </c>
       <c r="B133" t="s">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="F133" s="13"/>
       <c r="G133" s="13"/>
@@ -4062,14 +4426,14 @@
     </row>
     <row r="134" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A134" s="2">
-        <f t="shared" si="4"/>
-        <v>129</v>
+        <f t="shared" si="2"/>
+        <v>133</v>
       </c>
       <c r="B134" t="s">
-        <v>86</v>
+        <v>64</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="F134" s="13"/>
       <c r="G134" s="13"/>
@@ -4078,14 +4442,14 @@
     </row>
     <row r="135" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A135" s="2">
-        <f t="shared" si="4"/>
-        <v>130</v>
+        <f t="shared" si="2"/>
+        <v>134</v>
       </c>
       <c r="B135" t="s">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="F135" s="13"/>
       <c r="G135" s="13"/>
@@ -4094,14 +4458,14 @@
     </row>
     <row r="136" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A136" s="2">
-        <f t="shared" si="4"/>
-        <v>131</v>
+        <f t="shared" si="2"/>
+        <v>135</v>
       </c>
       <c r="B136" t="s">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>88</v>
+        <v>67</v>
       </c>
       <c r="F136" s="13"/>
       <c r="G136" s="13"/>
@@ -4110,43 +4474,343 @@
     </row>
     <row r="137" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A137" s="2">
-        <f t="shared" si="4"/>
-        <v>132</v>
+        <f t="shared" si="2"/>
+        <v>136</v>
       </c>
       <c r="B137" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="F137" s="13"/>
       <c r="G137" s="13"/>
       <c r="H137" s="11"/>
       <c r="I137" s="11"/>
     </row>
-    <row r="138" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="139" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="140" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="141" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="142" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="143" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="144" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="145" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="146" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="147" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="148" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="149" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="150" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="151" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="152" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="153" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="154" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="155" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="156" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="157" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="158" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="159" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="160" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="138" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A138" s="2">
+        <f t="shared" si="2"/>
+        <v>137</v>
+      </c>
+      <c r="B138" t="s">
+        <v>68</v>
+      </c>
+      <c r="C138" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F138" s="13"/>
+      <c r="G138" s="13"/>
+      <c r="H138" s="11"/>
+      <c r="I138" s="11"/>
+    </row>
+    <row r="139" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A139" s="2">
+        <f t="shared" si="2"/>
+        <v>138</v>
+      </c>
+      <c r="B139" t="s">
+        <v>68</v>
+      </c>
+      <c r="C139" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F139" s="13"/>
+      <c r="G139" s="13"/>
+      <c r="H139" s="11"/>
+      <c r="I139" s="11"/>
+    </row>
+    <row r="140" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A140" s="2">
+        <f t="shared" si="2"/>
+        <v>139</v>
+      </c>
+      <c r="B140" t="s">
+        <v>69</v>
+      </c>
+      <c r="C140" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F140" s="13"/>
+      <c r="G140" s="13"/>
+      <c r="H140" s="11"/>
+      <c r="I140" s="11"/>
+    </row>
+    <row r="141" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A141" s="2">
+        <f t="shared" si="2"/>
+        <v>140</v>
+      </c>
+      <c r="B141" t="s">
+        <v>69</v>
+      </c>
+      <c r="C141" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F141" s="13"/>
+      <c r="G141" s="13"/>
+      <c r="H141" s="11"/>
+      <c r="I141" s="11"/>
+    </row>
+    <row r="142" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A142" s="2">
+        <f t="shared" si="2"/>
+        <v>141</v>
+      </c>
+      <c r="B142" t="s">
+        <v>69</v>
+      </c>
+      <c r="C142" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F142" s="13"/>
+      <c r="G142" s="13"/>
+      <c r="H142" s="11"/>
+      <c r="I142" s="11"/>
+    </row>
+    <row r="143" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A143" s="2">
+        <f t="shared" si="2"/>
+        <v>142</v>
+      </c>
+      <c r="B143" t="s">
+        <v>73</v>
+      </c>
+      <c r="C143" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F143" s="13"/>
+      <c r="G143" s="13"/>
+      <c r="H143" s="11"/>
+      <c r="I143" s="11"/>
+    </row>
+    <row r="144" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A144" s="2">
+        <f t="shared" si="2"/>
+        <v>143</v>
+      </c>
+      <c r="B144" t="s">
+        <v>73</v>
+      </c>
+      <c r="C144" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F144" s="13"/>
+      <c r="G144" s="13"/>
+      <c r="H144" s="11"/>
+      <c r="I144" s="11"/>
+    </row>
+    <row r="145" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A145" s="2">
+        <f t="shared" si="2"/>
+        <v>144</v>
+      </c>
+      <c r="B145" t="s">
+        <v>73</v>
+      </c>
+      <c r="C145" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F145" s="13"/>
+      <c r="G145" s="13"/>
+      <c r="H145" s="11"/>
+      <c r="I145" s="11"/>
+    </row>
+    <row r="146" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A146" s="2">
+        <f t="shared" si="2"/>
+        <v>145</v>
+      </c>
+      <c r="B146" t="s">
+        <v>77</v>
+      </c>
+      <c r="C146" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F146" s="13"/>
+      <c r="G146" s="13"/>
+      <c r="H146" s="11"/>
+      <c r="I146" s="11"/>
+    </row>
+    <row r="147" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A147" s="2">
+        <f t="shared" si="2"/>
+        <v>146</v>
+      </c>
+      <c r="B147" t="s">
+        <v>77</v>
+      </c>
+      <c r="C147" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F147" s="13"/>
+      <c r="G147" s="13"/>
+      <c r="H147" s="11"/>
+      <c r="I147" s="11"/>
+    </row>
+    <row r="148" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A148" s="2">
+        <f t="shared" si="2"/>
+        <v>147</v>
+      </c>
+      <c r="B148" t="s">
+        <v>77</v>
+      </c>
+      <c r="C148" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F148" s="13"/>
+      <c r="G148" s="13"/>
+      <c r="H148" s="11"/>
+      <c r="I148" s="11"/>
+    </row>
+    <row r="149" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A149" s="2">
+        <f t="shared" si="2"/>
+        <v>148</v>
+      </c>
+      <c r="B149" t="s">
+        <v>78</v>
+      </c>
+      <c r="C149" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F149" s="13"/>
+      <c r="G149" s="13"/>
+      <c r="H149" s="11"/>
+      <c r="I149" s="11"/>
+    </row>
+    <row r="150" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A150" s="2">
+        <f t="shared" si="2"/>
+        <v>149</v>
+      </c>
+      <c r="B150" t="s">
+        <v>78</v>
+      </c>
+      <c r="C150" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F150" s="13"/>
+      <c r="G150" s="13"/>
+      <c r="H150" s="11"/>
+      <c r="I150" s="11"/>
+    </row>
+    <row r="151" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A151" s="2">
+        <f t="shared" si="2"/>
+        <v>150</v>
+      </c>
+      <c r="B151" t="s">
+        <v>78</v>
+      </c>
+      <c r="C151" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F151" s="13"/>
+      <c r="G151" s="13"/>
+      <c r="H151" s="11"/>
+      <c r="I151" s="11"/>
+    </row>
+    <row r="152" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A152" s="2">
+        <f t="shared" si="2"/>
+        <v>151</v>
+      </c>
+      <c r="B152" t="s">
+        <v>81</v>
+      </c>
+      <c r="C152" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F152" s="13"/>
+      <c r="G152" s="13"/>
+      <c r="H152" s="11"/>
+      <c r="I152" s="11"/>
+    </row>
+    <row r="153" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A153" s="2">
+        <f t="shared" si="2"/>
+        <v>152</v>
+      </c>
+      <c r="B153" t="s">
+        <v>81</v>
+      </c>
+      <c r="C153" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F153" s="13"/>
+      <c r="G153" s="13"/>
+      <c r="H153" s="11"/>
+      <c r="I153" s="11"/>
+    </row>
+    <row r="154" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A154" s="2">
+        <f t="shared" si="2"/>
+        <v>153</v>
+      </c>
+      <c r="B154" t="s">
+        <v>81</v>
+      </c>
+      <c r="C154" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F154" s="13"/>
+      <c r="G154" s="13"/>
+      <c r="H154" s="11"/>
+      <c r="I154" s="11"/>
+    </row>
+    <row r="155" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A155" s="2">
+        <f t="shared" si="2"/>
+        <v>154</v>
+      </c>
+      <c r="B155" t="s">
+        <v>85</v>
+      </c>
+      <c r="C155" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F155" s="13"/>
+      <c r="G155" s="13"/>
+      <c r="H155" s="11"/>
+      <c r="I155" s="11"/>
+    </row>
+    <row r="156" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A156" s="2">
+        <f t="shared" si="2"/>
+        <v>155</v>
+      </c>
+      <c r="B156" t="s">
+        <v>85</v>
+      </c>
+      <c r="C156" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F156" s="13"/>
+      <c r="G156" s="13"/>
+      <c r="H156" s="11"/>
+      <c r="I156" s="11"/>
+    </row>
+    <row r="157" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A157" s="2">
+        <f t="shared" ref="A157" si="3">A156+1</f>
+        <v>156</v>
+      </c>
+      <c r="B157" t="s">
+        <v>85</v>
+      </c>
+      <c r="C157" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F157" s="13"/>
+      <c r="G157" s="13"/>
+      <c r="H157" s="11"/>
+      <c r="I157" s="11"/>
+    </row>
+    <row r="158" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="159" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="160" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="161" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="162" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="163" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -4174,8 +4838,28 @@
     <row r="185" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="186" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="187" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="188" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="189" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="190" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="191" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="192" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="193" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="194" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="195" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="196" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="197" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="198" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="199" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="200" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="201" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="202" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="203" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="204" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="205" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="206" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="207" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>
-  <conditionalFormatting sqref="D2:D13 D15:D16 D18:D19 D21:D70 D72:D137">
+  <conditionalFormatting sqref="D2:D13 D15:D16 D18:D19 D21:D70 D72:D157">
     <cfRule type="cellIs" dxfId="9" priority="9" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -4216,7 +4900,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D149" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D169" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Pass,Fail"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add Neon palette and improve Ocean palette
- Enhanced Ocean palette with green/teal tones for more realistic ocean colors
- Added new Neon palette with high-frequency color cycling for detail revelation
- Neon uses rapid sine waves (16, 19, 23 Hz) with intensity boost for electric effect
- Alphabetized palette names in UI for better usability
- Fixed palette enum routing through managed/native bridge
- Added Neon = 7 to ColorPalette enum in FractalEngineWrapper.h
- Added Neon case to ParsePalette string-to-enum conversion
</commit_message>
<xml_diff>
--- a/ManpWinUI/Documentation/Architecture/PHASE5_STEP5.6_TEST_RESULTS.xlsx
+++ b/ManpWinUI/Documentation/Architecture/PHASE5_STEP5.6_TEST_RESULTS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\source\repos\ManpLab\ManpWinUI\Documentation\Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9C0AA9F-B103-41FA-A87F-EBCEE7775CD1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E36A2FB6-0307-49E9-8FA1-F5DA1051D3FD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="30720" windowHeight="12270" tabRatio="373" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,15 +16,15 @@
     <sheet name="PHASE5_STEP5.6_TEST_RESULTS" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PHASE5_STEP5.6_TEST_RESULTS!$A$1:$E$156</definedName>
-    <definedName name="Data">PHASE5_STEP5.6_TEST_RESULTS!$A$1:$I$156</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PHASE5_STEP5.6_TEST_RESULTS!$A$1:$I$157</definedName>
+    <definedName name="Data">PHASE5_STEP5.6_TEST_RESULTS!$A$1:$I$157</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="194">
   <si>
     <t>Group Name</t>
   </si>
@@ -3907,10 +3907,21 @@
       <c r="C101" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F101" s="13"/>
-      <c r="G101" s="13"/>
-      <c r="H101" s="11"/>
-      <c r="I101" s="11"/>
+      <c r="D101" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F101" s="13">
+        <v>0</v>
+      </c>
+      <c r="G101" s="13">
+        <v>5.75</v>
+      </c>
+      <c r="H101" s="11">
+        <v>19.607041454000001</v>
+      </c>
+      <c r="I101" s="11">
+        <v>11.028960818</v>
+      </c>
     </row>
     <row r="102" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A102" s="2">
@@ -4859,6 +4870,7 @@
     <row r="206" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="207" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>
+  <autoFilter ref="A1:I157" xr:uid="{53B5725F-EA7B-4922-8CC3-F684A90DDE36}"/>
   <conditionalFormatting sqref="D2:D13 D15:D16 D18:D19 D21:D70 D72:D157">
     <cfRule type="cellIs" dxfId="9" priority="9" operator="equal">
       <formula>"Fail"</formula>

</xml_diff>

<commit_message>
Update Phase 5 Step 5.6 test results
- Update test results spreadsheet with latest verification data
- Document fractal registry validation and naming conflict resolutions
</commit_message>
<xml_diff>
--- a/ManpWinUI/Documentation/Architecture/PHASE5_STEP5.6_TEST_RESULTS.xlsx
+++ b/ManpWinUI/Documentation/Architecture/PHASE5_STEP5.6_TEST_RESULTS.xlsx
@@ -8,23 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\source\repos\ManpLab\ManpWinUI\Documentation\Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E36A2FB6-0307-49E9-8FA1-F5DA1051D3FD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6017B8B-0297-4D6E-A842-08C8265B82C7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="30720" windowHeight="12270" tabRatio="373" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PHASE5_STEP5.6_TEST_RESULTS" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PHASE5_STEP5.6_TEST_RESULTS!$A$1:$I$157</definedName>
-    <definedName name="Data">PHASE5_STEP5.6_TEST_RESULTS!$A$1:$I$157</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PHASE5_STEP5.6_TEST_RESULTS!$A$1:$I$219</definedName>
+    <definedName name="Data">PHASE5_STEP5.6_TEST_RESULTS!$A$1:$I$219</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="252">
   <si>
     <t>Group Name</t>
   </si>
@@ -95,78 +97,24 @@
     <t>Hybrid Fractals</t>
   </si>
   <si>
-    <t>IFS</t>
-  </si>
-  <si>
-    <t>BarnsleyFern</t>
-  </si>
-  <si>
-    <t>DragonCurveIFS</t>
-  </si>
-  <si>
-    <t>PentagonIFS</t>
-  </si>
-  <si>
     <t>Julia Presets</t>
   </si>
   <si>
-    <t>Julia_Airplane</t>
-  </si>
-  <si>
-    <t>Julia_Backbone</t>
-  </si>
-  <si>
-    <t>Julia_Cauliflower</t>
-  </si>
-  <si>
     <t>Julia Sets</t>
   </si>
   <si>
-    <t>Julia4</t>
-  </si>
-  <si>
-    <t>Julia5</t>
-  </si>
-  <si>
-    <t>Julia6</t>
-  </si>
-  <si>
     <t>Lambda Fractals</t>
   </si>
   <si>
     <t>Lambda</t>
   </si>
   <si>
-    <t>LambdaFlip</t>
-  </si>
-  <si>
-    <t>LambdaJulia</t>
-  </si>
-  <si>
     <t>Magnet Fractals</t>
   </si>
   <si>
-    <t>Magnet1J</t>
-  </si>
-  <si>
-    <t>Magnet1M</t>
-  </si>
-  <si>
-    <t>Magnet1Power3</t>
-  </si>
-  <si>
     <t>Mandelbrot Variants</t>
   </si>
   <si>
-    <t>Buffalo</t>
-  </si>
-  <si>
-    <t>Celtic</t>
-  </si>
-  <si>
-    <t>Mandel4</t>
-  </si>
-  <si>
     <t>Newton's Method</t>
   </si>
   <si>
@@ -606,6 +554,234 @@
   </si>
   <si>
     <t>Trig-Mandelbrot Blend</t>
+  </si>
+  <si>
+    <t>Barnsley Fern (IFS)</t>
+  </si>
+  <si>
+    <t>Dragon Curve (IFS)</t>
+  </si>
+  <si>
+    <t>Pentagon (IFS)</t>
+  </si>
+  <si>
+    <t>Sierpinski Triangle (IFS)</t>
+  </si>
+  <si>
+    <t>Tree (IFS)</t>
+  </si>
+  <si>
+    <t>Iterated Function Systems</t>
+  </si>
+  <si>
+    <t>Julia - Airplane</t>
+  </si>
+  <si>
+    <t>Julia - Backbone</t>
+  </si>
+  <si>
+    <t>Julia - Cauliflower</t>
+  </si>
+  <si>
+    <t>Julia - Crystal</t>
+  </si>
+  <si>
+    <t>Julia - Dendrite</t>
+  </si>
+  <si>
+    <t>Julia - Dragon</t>
+  </si>
+  <si>
+    <t>Julia - Eye</t>
+  </si>
+  <si>
+    <t>Julia - Feigenbaum Point</t>
+  </si>
+  <si>
+    <t>Julia - Flower</t>
+  </si>
+  <si>
+    <t>Julia - Fractal Tree</t>
+  </si>
+  <si>
+    <t>Julia - Fuzzy Blob</t>
+  </si>
+  <si>
+    <t>Julia - Golden Ratio</t>
+  </si>
+  <si>
+    <t>Julia - Heart</t>
+  </si>
+  <si>
+    <t>Julia - Lightning</t>
+  </si>
+  <si>
+    <t>Julia - Medusa</t>
+  </si>
+  <si>
+    <t>Julia - Neurons</t>
+  </si>
+  <si>
+    <t>Julia - Paisley</t>
+  </si>
+  <si>
+    <t>Julia - Seahorse Valley</t>
+  </si>
+  <si>
+    <t>Julia - Snowflake</t>
+  </si>
+  <si>
+    <t>Julia - Spiral</t>
+  </si>
+  <si>
+    <t>Julia - Spiral Galaxy</t>
+  </si>
+  <si>
+    <t>Julia - Triple Spiral</t>
+  </si>
+  <si>
+    <t>Julia - Twisted Cross</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
+    <t>Douady Rabbit</t>
+  </si>
+  <si>
+    <t>San Marco</t>
+  </si>
+  <si>
+    <t>Siegel Disk</t>
+  </si>
+  <si>
+    <t>Burning Ship</t>
+  </si>
+  <si>
+    <t>Classic</t>
+  </si>
+  <si>
+    <t>Cubic</t>
+  </si>
+  <si>
+    <t>Exponential</t>
+  </si>
+  <si>
+    <t>Magnet</t>
+  </si>
+  <si>
+    <t>Lambda Julia</t>
+  </si>
+  <si>
+    <t>Sine</t>
+  </si>
+  <si>
+    <t>Multibrot 3</t>
+  </si>
+  <si>
+    <t>Multibrot 4</t>
+  </si>
+  <si>
+    <t>Power 5</t>
+  </si>
+  <si>
+    <t>Power 6</t>
+  </si>
+  <si>
+    <t>Julia - Burning Ship</t>
+  </si>
+  <si>
+    <t>Julia - Classic</t>
+  </si>
+  <si>
+    <t>Julia - Cubic</t>
+  </si>
+  <si>
+    <t>Julia - Custom</t>
+  </si>
+  <si>
+    <t>Julia - Douady Rabbit</t>
+  </si>
+  <si>
+    <t>Julia - Exponential</t>
+  </si>
+  <si>
+    <t>Julia - Lambda</t>
+  </si>
+  <si>
+    <t>Julia - Lambda (Alt)</t>
+  </si>
+  <si>
+    <t>Julia - Magnet</t>
+  </si>
+  <si>
+    <t>Julia - Multibrot 3</t>
+  </si>
+  <si>
+    <t>Julia - Multibrot 4</t>
+  </si>
+  <si>
+    <t>Julia - Phoenix</t>
+  </si>
+  <si>
+    <t>Julia - Power 5</t>
+  </si>
+  <si>
+    <t>Julia - Power 6</t>
+  </si>
+  <si>
+    <t>Julia - San Marco</t>
+  </si>
+  <si>
+    <t>Julia - Siegel Disk</t>
+  </si>
+  <si>
+    <t>Julia - Sine</t>
+  </si>
+  <si>
+    <t>Lambda Flip</t>
+  </si>
+  <si>
+    <t>Lambda Modified</t>
+  </si>
+  <si>
+    <t>Lambda Phoenix</t>
+  </si>
+  <si>
+    <t>Lambda Power 3</t>
+  </si>
+  <si>
+    <t>Lambda Power 4</t>
+  </si>
+  <si>
+    <t>Lambda Squared</t>
+  </si>
+  <si>
+    <t>Lambda Tan</t>
+  </si>
+  <si>
+    <t>Lambda Tanh</t>
+  </si>
+  <si>
+    <t>Magnet I Cubic</t>
+  </si>
+  <si>
+    <t>Magnet I Julia</t>
+  </si>
+  <si>
+    <t>Magnet II Cubic</t>
+  </si>
+  <si>
+    <t>Magnet II Julia</t>
+  </si>
+  <si>
+    <t>Celtic Heart</t>
+  </si>
+  <si>
+    <t>34 groups</t>
+  </si>
+  <si>
+    <t>294 fractals</t>
   </si>
 </sst>
 </file>
@@ -1127,7 +1303,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1179,6 +1355,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1605,7 +1783,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I207"/>
+  <dimension ref="A1:I269"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5.796875" style="2" customWidth="1"/>
@@ -1622,7 +1800,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="20.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" s="10" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>0</v>
@@ -1634,19 +1812,19 @@
         <v>2</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>111</v>
+        <v>93</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>112</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
@@ -1657,10 +1835,10 @@
         <v>3</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F2" s="13"/>
       <c r="G2" s="13"/>
@@ -1676,10 +1854,10 @@
         <v>3</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F3" s="13"/>
       <c r="G3" s="13"/>
@@ -1695,10 +1873,10 @@
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F4" s="13"/>
       <c r="G4" s="13"/>
@@ -1714,10 +1892,10 @@
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F5" s="13"/>
       <c r="G5" s="13"/>
@@ -1733,10 +1911,10 @@
         <v>3</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F6" s="13"/>
       <c r="G6" s="13"/>
@@ -1752,10 +1930,10 @@
         <v>3</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
@@ -1771,10 +1949,10 @@
         <v>3</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" s="14"/>
@@ -1791,10 +1969,10 @@
         <v>5</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F9" s="13"/>
       <c r="G9" s="13"/>
@@ -1810,10 +1988,10 @@
         <v>5</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F10" s="13"/>
       <c r="G10" s="13"/>
@@ -1829,10 +2007,10 @@
         <v>5</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
@@ -1848,10 +2026,10 @@
         <v>5</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F12" s="13"/>
       <c r="G12" s="13"/>
@@ -1867,10 +2045,10 @@
         <v>5</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
@@ -1886,10 +2064,10 @@
         <v>5</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="14"/>
@@ -1906,10 +2084,10 @@
         <v>6</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
@@ -1925,10 +2103,10 @@
         <v>6</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F16" s="13"/>
       <c r="G16" s="13"/>
@@ -1944,13 +2122,13 @@
         <v>6</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="F17" s="13"/>
       <c r="G17" s="13"/>
@@ -1966,10 +2144,10 @@
         <v>6</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E18" s="8"/>
       <c r="F18" s="13"/>
@@ -1986,13 +2164,13 @@
         <v>6</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="F19" s="13"/>
       <c r="G19" s="13"/>
@@ -2008,10 +2186,10 @@
         <v>6</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E20" s="6"/>
       <c r="F20" s="14"/>
@@ -2028,10 +2206,10 @@
         <v>7</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>113</v>
+        <v>95</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F21" s="13"/>
       <c r="G21" s="13"/>
@@ -2047,10 +2225,10 @@
         <v>7</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>187</v>
+        <v>169</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E22" s="6"/>
       <c r="F22" s="14"/>
@@ -2067,10 +2245,10 @@
         <v>8</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>114</v>
+        <v>96</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F23" s="13"/>
       <c r="G23" s="13"/>
@@ -2086,10 +2264,10 @@
         <v>8</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F24" s="13"/>
       <c r="G24" s="13"/>
@@ -2105,10 +2283,10 @@
         <v>8</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F25" s="13"/>
       <c r="G25" s="13"/>
@@ -2124,10 +2302,10 @@
         <v>8</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>117</v>
+        <v>99</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F26" s="13"/>
       <c r="G26" s="13"/>
@@ -2143,10 +2321,10 @@
         <v>8</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F27" s="13"/>
       <c r="G27" s="13"/>
@@ -2162,10 +2340,10 @@
         <v>8</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F28" s="13"/>
       <c r="G28" s="13"/>
@@ -2181,10 +2359,10 @@
         <v>8</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F29" s="13"/>
       <c r="G29" s="13"/>
@@ -2200,10 +2378,10 @@
         <v>8</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F30" s="13"/>
       <c r="G30" s="13"/>
@@ -2219,10 +2397,10 @@
         <v>8</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F31" s="13"/>
       <c r="G31" s="13"/>
@@ -2238,10 +2416,10 @@
         <v>8</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F32" s="13"/>
       <c r="G32" s="13"/>
@@ -2257,10 +2435,10 @@
         <v>8</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F33" s="13"/>
       <c r="G33" s="13"/>
@@ -2276,13 +2454,13 @@
         <v>8</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>126</v>
+        <v>108</v>
       </c>
       <c r="F34" s="14"/>
       <c r="G34" s="14"/>
@@ -2301,7 +2479,7 @@
         <v>4</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F35" s="13">
         <v>0</v>
@@ -2328,7 +2506,7 @@
         <v>10</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F36" s="13">
         <v>0</v>
@@ -2355,7 +2533,7 @@
         <v>11</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F37" s="13"/>
       <c r="G37" s="13"/>
@@ -2371,10 +2549,10 @@
         <v>9</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E38" s="6"/>
       <c r="F38" s="14"/>
@@ -2391,13 +2569,13 @@
         <v>12</v>
       </c>
       <c r="C39" s="17" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>186</v>
+        <v>168</v>
       </c>
       <c r="F39" s="15">
         <v>1</v>
@@ -2424,7 +2602,7 @@
         <v>13</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F40" s="13"/>
       <c r="G40" s="13"/>
@@ -2440,10 +2618,10 @@
         <v>12</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F41" s="13">
         <v>-1.5</v>
@@ -2467,10 +2645,10 @@
         <v>12</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E42" s="6"/>
       <c r="F42" s="14"/>
@@ -2487,10 +2665,10 @@
         <v>15</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F43" s="13"/>
       <c r="G43" s="13"/>
@@ -2506,10 +2684,10 @@
         <v>15</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>131</v>
+        <v>113</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F44" s="13"/>
       <c r="G44" s="13"/>
@@ -2525,10 +2703,10 @@
         <v>15</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F45" s="13"/>
       <c r="G45" s="13"/>
@@ -2544,10 +2722,10 @@
         <v>15</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>133</v>
+        <v>115</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F46" s="13"/>
       <c r="G46" s="13"/>
@@ -2563,10 +2741,10 @@
         <v>15</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F47" s="13"/>
       <c r="G47" s="13"/>
@@ -2582,10 +2760,10 @@
         <v>15</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>135</v>
+        <v>117</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F48" s="13"/>
       <c r="G48" s="13"/>
@@ -2601,10 +2779,10 @@
         <v>15</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E49" s="6"/>
       <c r="F49" s="14"/>
@@ -2621,10 +2799,10 @@
         <v>16</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>137</v>
+        <v>119</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F50" s="13"/>
       <c r="G50" s="13"/>
@@ -2640,10 +2818,10 @@
         <v>16</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>138</v>
+        <v>120</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F51" s="13"/>
       <c r="G51" s="13"/>
@@ -2659,10 +2837,10 @@
         <v>16</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>139</v>
+        <v>121</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F52" s="13"/>
       <c r="G52" s="13"/>
@@ -2678,10 +2856,10 @@
         <v>16</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>140</v>
+        <v>122</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E53" s="6"/>
       <c r="F53" s="14"/>
@@ -2698,10 +2876,10 @@
         <v>17</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>141</v>
+        <v>123</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F54" s="13">
         <v>-0.5</v>
@@ -2725,10 +2903,10 @@
         <v>17</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F55" s="13">
         <v>-0.6</v>
@@ -2752,10 +2930,10 @@
         <v>17</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>143</v>
+        <v>125</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F56" s="13">
         <v>-0.4</v>
@@ -2779,10 +2957,10 @@
         <v>17</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>144</v>
+        <v>126</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F57" s="13">
         <v>-0.8</v>
@@ -2806,10 +2984,10 @@
         <v>17</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>145</v>
+        <v>127</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F58" s="13">
         <v>-0.5</v>
@@ -2833,43 +3011,44 @@
         <v>17</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>146</v>
+        <v>128</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>147</v>
+        <v>129</v>
       </c>
       <c r="F59" s="13"/>
       <c r="G59" s="13"/>
       <c r="H59" s="11"/>
       <c r="I59" s="11"/>
     </row>
-    <row r="60" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:9" ht="20.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A60" s="2">
         <f t="shared" si="0"/>
         <v>59</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B60" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C60" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F60" s="13">
+      <c r="C60" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E60" s="6"/>
+      <c r="F60" s="14">
         <v>0</v>
       </c>
-      <c r="G60" s="13">
+      <c r="G60" s="14">
         <v>0</v>
       </c>
-      <c r="H60" s="11">
+      <c r="H60" s="12">
         <v>0.51202902653000004</v>
       </c>
-      <c r="I60" s="11">
+      <c r="I60" s="12">
         <v>0.28801632742</v>
       </c>
     </row>
@@ -2882,10 +3061,10 @@
         <v>18</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>149</v>
+        <v>131</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F61" s="13">
         <v>-0.5</v>
@@ -2909,10 +3088,10 @@
         <v>18</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>150</v>
+        <v>132</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
     </row>
     <row r="63" spans="1:9" ht="20.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
@@ -2924,10 +3103,10 @@
         <v>18</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>151</v>
+        <v>133</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E63" s="6"/>
       <c r="F63" s="14">
@@ -2952,10 +3131,10 @@
         <v>19</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>152</v>
+        <v>134</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F64" s="13">
         <v>0.5</v>
@@ -2979,10 +3158,10 @@
         <v>19</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>153</v>
+        <v>135</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F65" s="13"/>
       <c r="G65" s="13"/>
@@ -2998,10 +3177,10 @@
         <v>19</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>154</v>
+        <v>136</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F66" s="13">
         <v>-1</v>
@@ -3025,10 +3204,10 @@
         <v>19</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>155</v>
+        <v>137</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F67" s="13"/>
       <c r="G67" s="13"/>
@@ -3037,17 +3216,17 @@
     </row>
     <row r="68" spans="1:9" ht="31.9" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A68" s="2">
-        <f t="shared" ref="A68:A131" si="1">A67+1</f>
+        <f t="shared" ref="A68:A193" si="1">A67+1</f>
         <v>67</v>
       </c>
       <c r="B68" t="s">
         <v>19</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>156</v>
+        <v>138</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F68" s="13">
         <v>-2.5</v>
@@ -3071,10 +3250,10 @@
         <v>19</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>157</v>
+        <v>139</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F69" s="13">
         <v>0</v>
@@ -3098,13 +3277,13 @@
         <v>19</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>158</v>
+        <v>140</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>188</v>
+        <v>170</v>
       </c>
       <c r="F70" s="13">
         <v>0.875</v>
@@ -3128,13 +3307,13 @@
         <v>19</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>159</v>
+        <v>141</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>189</v>
+        <v>171</v>
       </c>
       <c r="F71" s="13">
         <v>0.24</v>
@@ -3158,10 +3337,10 @@
         <v>19</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>160</v>
+        <v>142</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F72" s="13">
         <v>-1.75</v>
@@ -3185,10 +3364,10 @@
         <v>19</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>161</v>
+        <v>143</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F73" s="13">
         <v>0.75</v>
@@ -3212,10 +3391,10 @@
         <v>19</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E74" s="6"/>
       <c r="F74" s="14">
@@ -3240,10 +3419,10 @@
         <v>20</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>164</v>
+        <v>146</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F75" s="13"/>
       <c r="G75" s="13"/>
@@ -3259,10 +3438,10 @@
         <v>20</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>163</v>
+        <v>145</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F76" s="13"/>
       <c r="G76" s="13"/>
@@ -3278,10 +3457,10 @@
         <v>20</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>165</v>
+        <v>147</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F77" s="13">
         <v>0</v>
@@ -3308,7 +3487,7 @@
         <v>21</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F78" s="13">
         <v>0</v>
@@ -3332,13 +3511,13 @@
         <v>20</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>166</v>
+        <v>148</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>167</v>
+        <v>149</v>
       </c>
       <c r="F79" s="13"/>
       <c r="G79" s="13"/>
@@ -3354,10 +3533,10 @@
         <v>20</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>168</v>
+        <v>150</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F80" s="13">
         <v>-0.75</v>
@@ -3381,10 +3560,10 @@
         <v>20</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>169</v>
+        <v>151</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F81" s="13"/>
       <c r="G81" s="13"/>
@@ -3400,10 +3579,10 @@
         <v>20</v>
       </c>
       <c r="C82" s="19" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
       <c r="D82" s="20" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E82" s="19"/>
       <c r="F82" s="21"/>
@@ -3420,10 +3599,10 @@
         <v>22</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>171</v>
+        <v>153</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F83" s="13">
         <v>1</v>
@@ -3447,10 +3626,10 @@
         <v>22</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>172</v>
+        <v>154</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F84" s="13">
         <v>-0.5</v>
@@ -3474,10 +3653,10 @@
         <v>22</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>141</v>
+        <v>123</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F85" s="13">
         <v>-0.75</v>
@@ -3501,10 +3680,10 @@
         <v>22</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>173</v>
+        <v>155</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F86" s="13">
         <v>-0.5</v>
@@ -3528,10 +3707,10 @@
         <v>22</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>174</v>
+        <v>156</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F87" s="13">
         <v>0</v>
@@ -3555,10 +3734,10 @@
         <v>22</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>175</v>
+        <v>157</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F88" s="13">
         <v>-1.4</v>
@@ -3582,10 +3761,10 @@
         <v>22</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>176</v>
+        <v>158</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F89" s="13">
         <v>-1.4</v>
@@ -3609,10 +3788,10 @@
         <v>22</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>177</v>
+        <v>159</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F90" s="13">
         <v>-2</v>
@@ -3636,10 +3815,10 @@
         <v>22</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F91" s="13">
         <v>0</v>
@@ -3663,10 +3842,10 @@
         <v>22</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>190</v>
+        <v>172</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F92" s="13">
         <v>-0.75</v>
@@ -3690,10 +3869,10 @@
         <v>22</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>179</v>
+        <v>161</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F93" s="13"/>
       <c r="G93" s="13"/>
@@ -3709,10 +3888,10 @@
         <v>22</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>180</v>
+        <v>162</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F94" s="13">
         <v>-0.5</v>
@@ -3736,13 +3915,13 @@
         <v>22</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>181</v>
+        <v>163</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>191</v>
+        <v>173</v>
       </c>
       <c r="F95" s="13">
         <v>-0.75</v>
@@ -3766,10 +3945,10 @@
         <v>22</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>182</v>
+        <v>164</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F96" s="13">
         <v>0</v>
@@ -3793,13 +3972,13 @@
         <v>22</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>192</v>
+        <v>174</v>
       </c>
       <c r="F97" s="13">
         <v>0</v>
@@ -3823,10 +4002,10 @@
         <v>22</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>184</v>
+        <v>166</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F98" s="13">
         <v>0</v>
@@ -3850,10 +4029,10 @@
         <v>22</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>185</v>
+        <v>167</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F99" s="13">
         <v>-0.58126820893451703</v>
@@ -3877,10 +4056,10 @@
         <v>22</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>193</v>
+        <v>175</v>
       </c>
       <c r="D100" s="5" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E100" s="6"/>
       <c r="F100" s="14">
@@ -3902,13 +4081,13 @@
         <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>23</v>
+        <v>181</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>24</v>
+        <v>176</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="F101" s="13">
         <v>0</v>
@@ -3929,15 +4108,26 @@
         <v>101</v>
       </c>
       <c r="B102" t="s">
-        <v>23</v>
+        <v>181</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F102" s="13"/>
-      <c r="G102" s="13"/>
-      <c r="H102" s="11"/>
-      <c r="I102" s="11"/>
+        <v>177</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F102" s="13">
+        <v>0.45753085666232601</v>
+      </c>
+      <c r="G102" s="13">
+        <v>0.18277777777777701</v>
+      </c>
+      <c r="H102" s="11">
+        <v>2.0306172839999999</v>
+      </c>
+      <c r="I102" s="11">
+        <v>1.1422222222</v>
+      </c>
     </row>
     <row r="103" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A103" s="2">
@@ -3945,15 +4135,26 @@
         <v>102</v>
       </c>
       <c r="B103" t="s">
-        <v>23</v>
+        <v>181</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F103" s="13"/>
-      <c r="G103" s="13"/>
-      <c r="H103" s="11"/>
-      <c r="I103" s="11"/>
+        <v>178</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F103" s="13">
+        <v>0</v>
+      </c>
+      <c r="G103" s="13">
+        <v>0</v>
+      </c>
+      <c r="H103" s="11">
+        <v>4</v>
+      </c>
+      <c r="I103" s="11">
+        <v>2.25</v>
+      </c>
     </row>
     <row r="104" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A104" s="2">
@@ -3961,31 +4162,54 @@
         <v>103</v>
       </c>
       <c r="B104" t="s">
-        <v>27</v>
+        <v>181</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F104" s="13"/>
-      <c r="G104" s="13"/>
-      <c r="H104" s="11"/>
-      <c r="I104" s="11"/>
-    </row>
-    <row r="105" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+        <v>179</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F104" s="13">
+        <v>0.5</v>
+      </c>
+      <c r="G104" s="13">
+        <v>0.433</v>
+      </c>
+      <c r="H104" s="11">
+        <v>2</v>
+      </c>
+      <c r="I104" s="11">
+        <v>1.125</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" ht="20.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A105" s="2">
         <f t="shared" si="1"/>
         <v>104</v>
       </c>
-      <c r="B105" t="s">
-        <v>27</v>
-      </c>
-      <c r="C105" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F105" s="13"/>
-      <c r="G105" s="13"/>
-      <c r="H105" s="11"/>
-      <c r="I105" s="11"/>
+      <c r="B105" s="23" t="s">
+        <v>181</v>
+      </c>
+      <c r="C105" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="D105" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E105" s="6"/>
+      <c r="F105" s="14">
+        <v>-5.3600823045271999E-3</v>
+      </c>
+      <c r="G105" s="14">
+        <v>1.0289157664609001</v>
+      </c>
+      <c r="H105" s="12">
+        <v>1.4744156379</v>
+      </c>
+      <c r="I105" s="12">
+        <v>0.82935879629999998</v>
+      </c>
     </row>
     <row r="106" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A106" s="2">
@@ -3993,15 +4217,26 @@
         <v>105</v>
       </c>
       <c r="B106" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F106" s="13"/>
-      <c r="G106" s="13"/>
-      <c r="H106" s="11"/>
-      <c r="I106" s="11"/>
+        <v>182</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F106" s="13">
+        <v>2.77704204776421E-2</v>
+      </c>
+      <c r="G106" s="13">
+        <v>-2.2920575359599699E-2</v>
+      </c>
+      <c r="H106" s="11">
+        <v>4.4267667291999997</v>
+      </c>
+      <c r="I106" s="11">
+        <v>2.4900562852000001</v>
+      </c>
     </row>
     <row r="107" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A107" s="2">
@@ -4009,15 +4244,26 @@
         <v>106</v>
       </c>
       <c r="B107" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F107" s="13"/>
-      <c r="G107" s="13"/>
-      <c r="H107" s="11"/>
-      <c r="I107" s="11"/>
+        <v>183</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F107" s="13">
+        <v>-7.6937178754299299E-2</v>
+      </c>
+      <c r="G107" s="13">
+        <v>9.1744840525328306E-3</v>
+      </c>
+      <c r="H107" s="11">
+        <v>4.0145090681999998</v>
+      </c>
+      <c r="I107" s="11">
+        <v>2.2581613508</v>
+      </c>
     </row>
     <row r="108" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A108" s="2">
@@ -4025,15 +4271,26 @@
         <v>107</v>
       </c>
       <c r="B108" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F108" s="13"/>
-      <c r="G108" s="13"/>
-      <c r="H108" s="11"/>
-      <c r="I108" s="11"/>
+        <v>184</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F108" s="13">
+        <v>-4.2501624550500203E-2</v>
+      </c>
+      <c r="G108" s="13">
+        <v>-1.49656035021887E-2</v>
+      </c>
+      <c r="H108" s="11">
+        <v>5.2552845528000001</v>
+      </c>
+      <c r="I108" s="11">
+        <v>2.956097561</v>
+      </c>
     </row>
     <row r="109" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A109" s="2">
@@ -4041,15 +4298,26 @@
         <v>108</v>
       </c>
       <c r="B109" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F109" s="13"/>
-      <c r="G109" s="13"/>
-      <c r="H109" s="11"/>
-      <c r="I109" s="11"/>
+        <v>185</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F109" s="13">
+        <v>0.20147063989522099</v>
+      </c>
+      <c r="G109" s="13">
+        <v>-2.16709757128607E-2</v>
+      </c>
+      <c r="H109" s="11">
+        <v>4.3163112450999996</v>
+      </c>
+      <c r="I109" s="11">
+        <v>2.4279250753000001</v>
+      </c>
     </row>
     <row r="110" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A110" s="2">
@@ -4057,10 +4325,10 @@
         <v>109</v>
       </c>
       <c r="B110" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>36</v>
+        <v>186</v>
       </c>
       <c r="F110" s="13"/>
       <c r="G110" s="13"/>
@@ -4073,10 +4341,10 @@
         <v>110</v>
       </c>
       <c r="B111" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>37</v>
+        <v>187</v>
       </c>
       <c r="F111" s="13"/>
       <c r="G111" s="13"/>
@@ -4089,10 +4357,10 @@
         <v>111</v>
       </c>
       <c r="B112" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>38</v>
+        <v>188</v>
       </c>
       <c r="F112" s="13"/>
       <c r="G112" s="13"/>
@@ -4105,10 +4373,10 @@
         <v>112</v>
       </c>
       <c r="B113" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>40</v>
+        <v>189</v>
       </c>
       <c r="F113" s="13"/>
       <c r="G113" s="13"/>
@@ -4121,10 +4389,10 @@
         <v>113</v>
       </c>
       <c r="B114" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>41</v>
+        <v>190</v>
       </c>
       <c r="F114" s="13"/>
       <c r="G114" s="13"/>
@@ -4137,10 +4405,10 @@
         <v>114</v>
       </c>
       <c r="B115" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>42</v>
+        <v>191</v>
       </c>
       <c r="F115" s="13"/>
       <c r="G115" s="13"/>
@@ -4153,10 +4421,10 @@
         <v>115</v>
       </c>
       <c r="B116" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>44</v>
+        <v>192</v>
       </c>
       <c r="F116" s="13"/>
       <c r="G116" s="13"/>
@@ -4169,10 +4437,10 @@
         <v>116</v>
       </c>
       <c r="B117" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>45</v>
+        <v>193</v>
       </c>
       <c r="F117" s="13"/>
       <c r="G117" s="13"/>
@@ -4185,10 +4453,10 @@
         <v>117</v>
       </c>
       <c r="B118" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>46</v>
+        <v>194</v>
       </c>
       <c r="F118" s="13"/>
       <c r="G118" s="13"/>
@@ -4201,10 +4469,10 @@
         <v>118</v>
       </c>
       <c r="B119" t="s">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>48</v>
+        <v>195</v>
       </c>
       <c r="F119" s="13"/>
       <c r="G119" s="13"/>
@@ -4217,10 +4485,10 @@
         <v>119</v>
       </c>
       <c r="B120" t="s">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>49</v>
+        <v>196</v>
       </c>
       <c r="F120" s="13"/>
       <c r="G120" s="13"/>
@@ -4233,10 +4501,10 @@
         <v>120</v>
       </c>
       <c r="B121" t="s">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>50</v>
+        <v>197</v>
       </c>
       <c r="F121" s="13"/>
       <c r="G121" s="13"/>
@@ -4249,10 +4517,10 @@
         <v>121</v>
       </c>
       <c r="B122" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>52</v>
+        <v>198</v>
       </c>
       <c r="F122" s="13"/>
       <c r="G122" s="13"/>
@@ -4265,10 +4533,10 @@
         <v>122</v>
       </c>
       <c r="B123" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>53</v>
+        <v>199</v>
       </c>
       <c r="F123" s="13"/>
       <c r="G123" s="13"/>
@@ -4281,10 +4549,10 @@
         <v>123</v>
       </c>
       <c r="B124" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>54</v>
+        <v>200</v>
       </c>
       <c r="F124" s="13"/>
       <c r="G124" s="13"/>
@@ -4297,10 +4565,10 @@
         <v>124</v>
       </c>
       <c r="B125" t="s">
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>52</v>
+        <v>201</v>
       </c>
       <c r="F125" s="13"/>
       <c r="G125" s="13"/>
@@ -4313,10 +4581,10 @@
         <v>125</v>
       </c>
       <c r="B126" t="s">
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>53</v>
+        <v>202</v>
       </c>
       <c r="F126" s="13"/>
       <c r="G126" s="13"/>
@@ -4329,314 +4597,350 @@
         <v>126</v>
       </c>
       <c r="B127" t="s">
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>54</v>
+        <v>203</v>
       </c>
       <c r="F127" s="13"/>
       <c r="G127" s="13"/>
       <c r="H127" s="11"/>
       <c r="I127" s="11"/>
     </row>
-    <row r="128" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="128" spans="1:9" ht="20.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A128" s="2">
         <f t="shared" si="1"/>
         <v>127</v>
       </c>
-      <c r="B128" t="s">
-        <v>56</v>
-      </c>
-      <c r="C128" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="F128" s="13"/>
-      <c r="G128" s="13"/>
-      <c r="H128" s="11"/>
-      <c r="I128" s="11"/>
+      <c r="B128" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C128" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="D128" s="5"/>
+      <c r="E128" s="6"/>
+      <c r="F128" s="14"/>
+      <c r="G128" s="14"/>
+      <c r="H128" s="12"/>
+      <c r="I128" s="12"/>
     </row>
     <row r="129" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A129" s="2">
         <f t="shared" si="1"/>
         <v>128</v>
       </c>
-      <c r="B129" t="s">
-        <v>56</v>
-      </c>
-      <c r="C129" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F129" s="13"/>
-      <c r="G129" s="13"/>
-      <c r="H129" s="11"/>
-      <c r="I129" s="11"/>
+      <c r="B129" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C129" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="D129" s="7"/>
+      <c r="E129" s="8"/>
+      <c r="F129" s="15"/>
+      <c r="G129" s="15"/>
+      <c r="H129" s="16"/>
+      <c r="I129" s="16"/>
     </row>
     <row r="130" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A130" s="2">
         <f t="shared" si="1"/>
         <v>129</v>
       </c>
-      <c r="B130" t="s">
-        <v>56</v>
-      </c>
-      <c r="C130" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="F130" s="13"/>
-      <c r="G130" s="13"/>
-      <c r="H130" s="11"/>
-      <c r="I130" s="11"/>
+      <c r="B130" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C130" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="D130" s="7"/>
+      <c r="E130" s="8"/>
+      <c r="F130" s="15"/>
+      <c r="G130" s="15"/>
+      <c r="H130" s="16"/>
+      <c r="I130" s="16"/>
     </row>
     <row r="131" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A131" s="2">
         <f t="shared" si="1"/>
         <v>130</v>
       </c>
-      <c r="B131" t="s">
-        <v>60</v>
-      </c>
-      <c r="C131" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="F131" s="13"/>
-      <c r="G131" s="13"/>
-      <c r="H131" s="11"/>
-      <c r="I131" s="11"/>
+      <c r="B131" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C131" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="D131" s="7"/>
+      <c r="E131" s="8"/>
+      <c r="F131" s="15"/>
+      <c r="G131" s="15"/>
+      <c r="H131" s="16"/>
+      <c r="I131" s="16"/>
     </row>
     <row r="132" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A132" s="2">
-        <f t="shared" ref="A132:A156" si="2">A131+1</f>
+        <f t="shared" si="1"/>
         <v>131</v>
       </c>
-      <c r="B132" t="s">
-        <v>60</v>
-      </c>
-      <c r="C132" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F132" s="13"/>
-      <c r="G132" s="13"/>
-      <c r="H132" s="11"/>
-      <c r="I132" s="11"/>
+      <c r="B132" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C132" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="D132" s="7"/>
+      <c r="E132" s="8"/>
+      <c r="F132" s="15"/>
+      <c r="G132" s="15"/>
+      <c r="H132" s="16"/>
+      <c r="I132" s="16"/>
     </row>
     <row r="133" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A133" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>132</v>
       </c>
-      <c r="B133" t="s">
-        <v>60</v>
-      </c>
-      <c r="C133" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F133" s="13"/>
-      <c r="G133" s="13"/>
-      <c r="H133" s="11"/>
-      <c r="I133" s="11"/>
+      <c r="B133" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C133" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="D133" s="7"/>
+      <c r="E133" s="8"/>
+      <c r="F133" s="15"/>
+      <c r="G133" s="15"/>
+      <c r="H133" s="16"/>
+      <c r="I133" s="16"/>
     </row>
     <row r="134" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A134" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>133</v>
       </c>
-      <c r="B134" t="s">
-        <v>64</v>
-      </c>
-      <c r="C134" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F134" s="13"/>
-      <c r="G134" s="13"/>
-      <c r="H134" s="11"/>
-      <c r="I134" s="11"/>
+      <c r="B134" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C134" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="D134" s="7"/>
+      <c r="E134" s="8"/>
+      <c r="F134" s="15"/>
+      <c r="G134" s="15"/>
+      <c r="H134" s="16"/>
+      <c r="I134" s="16"/>
     </row>
     <row r="135" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A135" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>134</v>
       </c>
-      <c r="B135" t="s">
-        <v>64</v>
-      </c>
-      <c r="C135" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F135" s="13"/>
-      <c r="G135" s="13"/>
-      <c r="H135" s="11"/>
-      <c r="I135" s="11"/>
+      <c r="B135" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C135" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="D135" s="7"/>
+      <c r="E135" s="8"/>
+      <c r="F135" s="15"/>
+      <c r="G135" s="15"/>
+      <c r="H135" s="16"/>
+      <c r="I135" s="16"/>
     </row>
     <row r="136" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A136" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>135</v>
       </c>
-      <c r="B136" t="s">
-        <v>64</v>
-      </c>
-      <c r="C136" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="F136" s="13"/>
-      <c r="G136" s="13"/>
-      <c r="H136" s="11"/>
-      <c r="I136" s="11"/>
+      <c r="B136" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C136" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="D136" s="7"/>
+      <c r="E136" s="8"/>
+      <c r="F136" s="15"/>
+      <c r="G136" s="15"/>
+      <c r="H136" s="16"/>
+      <c r="I136" s="16"/>
     </row>
     <row r="137" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A137" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>136</v>
       </c>
-      <c r="B137" t="s">
-        <v>68</v>
-      </c>
-      <c r="C137" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F137" s="13"/>
-      <c r="G137" s="13"/>
-      <c r="H137" s="11"/>
-      <c r="I137" s="11"/>
+      <c r="B137" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C137" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="D137" s="7"/>
+      <c r="E137" s="8"/>
+      <c r="F137" s="15"/>
+      <c r="G137" s="15"/>
+      <c r="H137" s="16"/>
+      <c r="I137" s="16"/>
     </row>
     <row r="138" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A138" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>137</v>
       </c>
-      <c r="B138" t="s">
-        <v>68</v>
-      </c>
-      <c r="C138" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F138" s="13"/>
-      <c r="G138" s="13"/>
-      <c r="H138" s="11"/>
-      <c r="I138" s="11"/>
+      <c r="B138" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C138" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="D138" s="7"/>
+      <c r="E138" s="8"/>
+      <c r="F138" s="15"/>
+      <c r="G138" s="15"/>
+      <c r="H138" s="16"/>
+      <c r="I138" s="16"/>
     </row>
     <row r="139" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A139" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>138</v>
       </c>
-      <c r="B139" t="s">
-        <v>68</v>
-      </c>
-      <c r="C139" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="F139" s="13"/>
-      <c r="G139" s="13"/>
-      <c r="H139" s="11"/>
-      <c r="I139" s="11"/>
+      <c r="B139" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C139" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="D139" s="7"/>
+      <c r="E139" s="8"/>
+      <c r="F139" s="15"/>
+      <c r="G139" s="15"/>
+      <c r="H139" s="16"/>
+      <c r="I139" s="16"/>
     </row>
     <row r="140" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A140" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>139</v>
       </c>
-      <c r="B140" t="s">
-        <v>69</v>
-      </c>
-      <c r="C140" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="F140" s="13"/>
-      <c r="G140" s="13"/>
-      <c r="H140" s="11"/>
-      <c r="I140" s="11"/>
+      <c r="B140" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C140" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="D140" s="7"/>
+      <c r="E140" s="8"/>
+      <c r="F140" s="15"/>
+      <c r="G140" s="15"/>
+      <c r="H140" s="16"/>
+      <c r="I140" s="16"/>
     </row>
     <row r="141" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A141" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>140</v>
       </c>
-      <c r="B141" t="s">
-        <v>69</v>
-      </c>
-      <c r="C141" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="F141" s="13"/>
-      <c r="G141" s="13"/>
-      <c r="H141" s="11"/>
-      <c r="I141" s="11"/>
+      <c r="B141" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C141" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="D141" s="7"/>
+      <c r="E141" s="8"/>
+      <c r="F141" s="15"/>
+      <c r="G141" s="15"/>
+      <c r="H141" s="16"/>
+      <c r="I141" s="16"/>
     </row>
     <row r="142" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A142" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>141</v>
       </c>
-      <c r="B142" t="s">
-        <v>69</v>
-      </c>
-      <c r="C142" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="F142" s="13"/>
-      <c r="G142" s="13"/>
-      <c r="H142" s="11"/>
-      <c r="I142" s="11"/>
+      <c r="B142" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C142" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="D142" s="7"/>
+      <c r="E142" s="8"/>
+      <c r="F142" s="15"/>
+      <c r="G142" s="15"/>
+      <c r="H142" s="16"/>
+      <c r="I142" s="16"/>
     </row>
     <row r="143" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A143" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>142</v>
       </c>
-      <c r="B143" t="s">
-        <v>73</v>
-      </c>
-      <c r="C143" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="F143" s="13"/>
-      <c r="G143" s="13"/>
-      <c r="H143" s="11"/>
-      <c r="I143" s="11"/>
+      <c r="B143" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C143" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="D143" s="7"/>
+      <c r="E143" s="8"/>
+      <c r="F143" s="15"/>
+      <c r="G143" s="15"/>
+      <c r="H143" s="16"/>
+      <c r="I143" s="16"/>
     </row>
     <row r="144" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A144" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>143</v>
       </c>
-      <c r="B144" t="s">
-        <v>73</v>
-      </c>
-      <c r="C144" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="F144" s="13"/>
-      <c r="G144" s="13"/>
-      <c r="H144" s="11"/>
-      <c r="I144" s="11"/>
-    </row>
-    <row r="145" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B144" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C144" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="D144" s="7"/>
+      <c r="E144" s="8"/>
+      <c r="F144" s="15"/>
+      <c r="G144" s="15"/>
+      <c r="H144" s="16"/>
+      <c r="I144" s="16"/>
+    </row>
+    <row r="145" spans="1:9" ht="20.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A145" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>144</v>
       </c>
-      <c r="B145" t="s">
-        <v>73</v>
-      </c>
-      <c r="C145" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="F145" s="13"/>
-      <c r="G145" s="13"/>
-      <c r="H145" s="11"/>
-      <c r="I145" s="11"/>
+      <c r="B145" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="C145" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="D145" s="5"/>
+      <c r="E145" s="6"/>
+      <c r="F145" s="14"/>
+      <c r="G145" s="14"/>
+      <c r="H145" s="12"/>
+      <c r="I145" s="12"/>
     </row>
     <row r="146" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A146" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>145</v>
       </c>
       <c r="B146" t="s">
-        <v>77</v>
+        <v>25</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>74</v>
+        <v>237</v>
       </c>
       <c r="F146" s="13"/>
       <c r="G146" s="13"/>
@@ -4645,14 +4949,14 @@
     </row>
     <row r="147" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A147" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>146</v>
       </c>
       <c r="B147" t="s">
-        <v>77</v>
+        <v>25</v>
       </c>
       <c r="C147" s="1" t="s">
-        <v>75</v>
+        <v>238</v>
       </c>
       <c r="F147" s="13"/>
       <c r="G147" s="13"/>
@@ -4661,14 +4965,14 @@
     </row>
     <row r="148" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A148" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>147</v>
       </c>
       <c r="B148" t="s">
-        <v>77</v>
+        <v>25</v>
       </c>
       <c r="C148" s="1" t="s">
-        <v>76</v>
+        <v>239</v>
       </c>
       <c r="F148" s="13"/>
       <c r="G148" s="13"/>
@@ -4677,14 +4981,14 @@
     </row>
     <row r="149" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A149" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>148</v>
       </c>
       <c r="B149" t="s">
-        <v>78</v>
+        <v>25</v>
       </c>
       <c r="C149" s="1" t="s">
-        <v>14</v>
+        <v>240</v>
       </c>
       <c r="F149" s="13"/>
       <c r="G149" s="13"/>
@@ -4693,14 +4997,14 @@
     </row>
     <row r="150" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A150" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>149</v>
       </c>
       <c r="B150" t="s">
-        <v>78</v>
+        <v>25</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>79</v>
+        <v>241</v>
       </c>
       <c r="F150" s="13"/>
       <c r="G150" s="13"/>
@@ -4709,14 +5013,14 @@
     </row>
     <row r="151" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A151" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>150</v>
       </c>
       <c r="B151" t="s">
-        <v>78</v>
+        <v>25</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>80</v>
+        <v>242</v>
       </c>
       <c r="F151" s="13"/>
       <c r="G151" s="13"/>
@@ -4725,62 +5029,62 @@
     </row>
     <row r="152" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A152" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>151</v>
       </c>
       <c r="B152" t="s">
-        <v>81</v>
+        <v>25</v>
       </c>
       <c r="C152" s="1" t="s">
-        <v>82</v>
+        <v>243</v>
       </c>
       <c r="F152" s="13"/>
       <c r="G152" s="13"/>
       <c r="H152" s="11"/>
       <c r="I152" s="11"/>
     </row>
-    <row r="153" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="153" spans="1:9" ht="20.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A153" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>152</v>
       </c>
-      <c r="B153" t="s">
-        <v>81</v>
-      </c>
-      <c r="C153" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F153" s="13"/>
-      <c r="G153" s="13"/>
-      <c r="H153" s="11"/>
-      <c r="I153" s="11"/>
+      <c r="B153" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C153" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="D153" s="5"/>
+      <c r="E153" s="6"/>
+      <c r="F153" s="14"/>
+      <c r="G153" s="14"/>
+      <c r="H153" s="12"/>
+      <c r="I153" s="12"/>
     </row>
     <row r="154" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A154" s="2">
-        <f t="shared" si="2"/>
-        <v>153</v>
-      </c>
-      <c r="B154" t="s">
-        <v>81</v>
-      </c>
-      <c r="C154" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="F154" s="13"/>
-      <c r="G154" s="13"/>
-      <c r="H154" s="11"/>
-      <c r="I154" s="11"/>
+      <c r="B154" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C154" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="D154" s="7"/>
+      <c r="E154" s="8"/>
+      <c r="F154" s="15"/>
+      <c r="G154" s="15"/>
+      <c r="H154" s="16"/>
+      <c r="I154" s="16"/>
     </row>
     <row r="155" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A155" s="2">
-        <f t="shared" si="2"/>
-        <v>154</v>
+        <f>A153+1</f>
+        <v>153</v>
       </c>
       <c r="B155" t="s">
-        <v>85</v>
+        <v>27</v>
       </c>
       <c r="C155" s="1" t="s">
-        <v>82</v>
+        <v>246</v>
       </c>
       <c r="F155" s="13"/>
       <c r="G155" s="13"/>
@@ -4789,89 +5093,907 @@
     </row>
     <row r="156" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A156" s="2">
-        <f t="shared" si="2"/>
-        <v>155</v>
+        <f t="shared" si="1"/>
+        <v>154</v>
       </c>
       <c r="B156" t="s">
-        <v>85</v>
+        <v>27</v>
       </c>
       <c r="C156" s="1" t="s">
-        <v>83</v>
+        <v>247</v>
       </c>
       <c r="F156" s="13"/>
       <c r="G156" s="13"/>
       <c r="H156" s="11"/>
       <c r="I156" s="11"/>
     </row>
-    <row r="157" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="157" spans="1:9" ht="20.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A157" s="2">
-        <f t="shared" ref="A157" si="3">A156+1</f>
+        <f t="shared" si="1"/>
+        <v>155</v>
+      </c>
+      <c r="B157" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C157" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="D157" s="5"/>
+      <c r="E157" s="6"/>
+      <c r="F157" s="14"/>
+      <c r="G157" s="14"/>
+      <c r="H157" s="12"/>
+      <c r="I157" s="12"/>
+    </row>
+    <row r="158" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A158" s="2">
+        <f t="shared" si="1"/>
         <v>156</v>
       </c>
-      <c r="B157" t="s">
-        <v>85</v>
-      </c>
-      <c r="C157" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="F157" s="13"/>
-      <c r="G157" s="13"/>
-      <c r="H157" s="11"/>
-      <c r="I157" s="11"/>
-    </row>
-    <row r="158" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="159" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="160" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="161" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="162" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="163" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="164" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="165" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="166" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="167" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="168" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="169" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="170" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="171" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="172" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="173" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="174" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="175" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="176" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="177" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="178" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="179" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="180" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="181" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="182" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="183" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="184" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="185" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="186" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="187" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="188" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="189" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="190" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="191" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="192" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="193" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="194" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="195" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="196" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="197" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="198" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="199" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="200" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="201" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="202" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="203" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="204" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="205" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="206" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="207" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+      <c r="B158" t="s">
+        <v>28</v>
+      </c>
+      <c r="C158" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="F158" s="13"/>
+      <c r="G158" s="13"/>
+      <c r="H158" s="11"/>
+      <c r="I158" s="11"/>
+    </row>
+    <row r="159" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A159" s="2">
+        <f t="shared" si="1"/>
+        <v>157</v>
+      </c>
+      <c r="B159" t="s">
+        <v>28</v>
+      </c>
+      <c r="C159" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="F159" s="13"/>
+      <c r="G159" s="13"/>
+      <c r="H159" s="11"/>
+      <c r="I159" s="11"/>
+    </row>
+    <row r="160" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C160" s="1"/>
+      <c r="F160" s="13"/>
+      <c r="G160" s="13"/>
+      <c r="H160" s="11"/>
+      <c r="I160" s="11"/>
+    </row>
+    <row r="161" spans="3:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C161" s="1"/>
+      <c r="F161" s="13"/>
+      <c r="G161" s="13"/>
+      <c r="H161" s="11"/>
+      <c r="I161" s="11"/>
+    </row>
+    <row r="162" spans="3:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C162" s="1"/>
+      <c r="F162" s="13"/>
+      <c r="G162" s="13"/>
+      <c r="H162" s="11"/>
+      <c r="I162" s="11"/>
+    </row>
+    <row r="163" spans="3:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C163" s="1"/>
+      <c r="F163" s="13"/>
+      <c r="G163" s="13"/>
+      <c r="H163" s="11"/>
+      <c r="I163" s="11"/>
+    </row>
+    <row r="164" spans="3:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C164" s="1"/>
+      <c r="F164" s="13"/>
+      <c r="G164" s="13"/>
+      <c r="H164" s="11"/>
+      <c r="I164" s="11"/>
+    </row>
+    <row r="165" spans="3:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C165" s="1"/>
+      <c r="F165" s="13"/>
+      <c r="G165" s="13"/>
+      <c r="H165" s="11"/>
+      <c r="I165" s="11"/>
+    </row>
+    <row r="166" spans="3:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C166" s="1"/>
+      <c r="F166" s="13"/>
+      <c r="G166" s="13"/>
+      <c r="H166" s="11"/>
+      <c r="I166" s="11"/>
+    </row>
+    <row r="167" spans="3:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C167" s="1"/>
+      <c r="F167" s="13"/>
+      <c r="G167" s="13"/>
+      <c r="H167" s="11"/>
+      <c r="I167" s="11"/>
+    </row>
+    <row r="168" spans="3:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C168" s="1"/>
+      <c r="F168" s="13"/>
+      <c r="G168" s="13"/>
+      <c r="H168" s="11"/>
+      <c r="I168" s="11"/>
+    </row>
+    <row r="169" spans="3:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C169" s="1"/>
+      <c r="F169" s="13"/>
+      <c r="G169" s="13"/>
+      <c r="H169" s="11"/>
+      <c r="I169" s="11"/>
+    </row>
+    <row r="170" spans="3:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C170" s="1"/>
+      <c r="F170" s="13"/>
+      <c r="G170" s="13"/>
+      <c r="H170" s="11"/>
+      <c r="I170" s="11"/>
+    </row>
+    <row r="171" spans="3:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C171" s="1"/>
+      <c r="F171" s="13"/>
+      <c r="G171" s="13"/>
+      <c r="H171" s="11"/>
+      <c r="I171" s="11"/>
+    </row>
+    <row r="172" spans="3:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C172" s="1"/>
+      <c r="F172" s="13"/>
+      <c r="G172" s="13"/>
+      <c r="H172" s="11"/>
+      <c r="I172" s="11"/>
+    </row>
+    <row r="173" spans="3:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C173" s="1"/>
+      <c r="F173" s="13"/>
+      <c r="G173" s="13"/>
+      <c r="H173" s="11"/>
+      <c r="I173" s="11"/>
+    </row>
+    <row r="174" spans="3:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C174" s="1"/>
+      <c r="F174" s="13"/>
+      <c r="G174" s="13"/>
+      <c r="H174" s="11"/>
+      <c r="I174" s="11"/>
+    </row>
+    <row r="175" spans="3:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C175" s="1"/>
+      <c r="F175" s="13"/>
+      <c r="G175" s="13"/>
+      <c r="H175" s="11"/>
+      <c r="I175" s="11"/>
+    </row>
+    <row r="176" spans="3:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C176" s="1"/>
+      <c r="F176" s="13"/>
+      <c r="G176" s="13"/>
+      <c r="H176" s="11"/>
+      <c r="I176" s="11"/>
+    </row>
+    <row r="177" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C177" s="1"/>
+      <c r="F177" s="13"/>
+      <c r="G177" s="13"/>
+      <c r="H177" s="11"/>
+      <c r="I177" s="11"/>
+    </row>
+    <row r="178" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C178" s="1"/>
+      <c r="F178" s="13"/>
+      <c r="G178" s="13"/>
+      <c r="H178" s="11"/>
+      <c r="I178" s="11"/>
+    </row>
+    <row r="179" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C179" s="1"/>
+      <c r="F179" s="13"/>
+      <c r="G179" s="13"/>
+      <c r="H179" s="11"/>
+      <c r="I179" s="11"/>
+    </row>
+    <row r="180" spans="1:9" ht="20.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A180" s="2">
+        <f>A159+1</f>
+        <v>158</v>
+      </c>
+      <c r="B180" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C180" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D180" s="5"/>
+      <c r="E180" s="6"/>
+      <c r="F180" s="14"/>
+      <c r="G180" s="14"/>
+      <c r="H180" s="12"/>
+      <c r="I180" s="12"/>
+    </row>
+    <row r="181" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A181" s="2">
+        <f t="shared" si="1"/>
+        <v>159</v>
+      </c>
+      <c r="B181" t="s">
+        <v>29</v>
+      </c>
+      <c r="C181" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F181" s="13"/>
+      <c r="G181" s="13"/>
+      <c r="H181" s="11"/>
+      <c r="I181" s="11"/>
+    </row>
+    <row r="182" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A182" s="2">
+        <f t="shared" si="1"/>
+        <v>160</v>
+      </c>
+      <c r="B182" t="s">
+        <v>29</v>
+      </c>
+      <c r="C182" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F182" s="13"/>
+      <c r="G182" s="13"/>
+      <c r="H182" s="11"/>
+      <c r="I182" s="11"/>
+    </row>
+    <row r="183" spans="1:9" ht="20.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A183" s="2">
+        <f t="shared" si="1"/>
+        <v>161</v>
+      </c>
+      <c r="B183" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C183" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D183" s="5"/>
+      <c r="E183" s="6"/>
+      <c r="F183" s="14"/>
+      <c r="G183" s="14"/>
+      <c r="H183" s="12"/>
+      <c r="I183" s="12"/>
+    </row>
+    <row r="184" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A184" s="2">
+        <f t="shared" si="1"/>
+        <v>162</v>
+      </c>
+      <c r="B184" t="s">
+        <v>33</v>
+      </c>
+      <c r="C184" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F184" s="13"/>
+      <c r="G184" s="13"/>
+      <c r="H184" s="11"/>
+      <c r="I184" s="11"/>
+    </row>
+    <row r="185" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A185" s="2">
+        <f t="shared" si="1"/>
+        <v>163</v>
+      </c>
+      <c r="B185" t="s">
+        <v>33</v>
+      </c>
+      <c r="C185" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F185" s="13"/>
+      <c r="G185" s="13"/>
+      <c r="H185" s="11"/>
+      <c r="I185" s="11"/>
+    </row>
+    <row r="186" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A186" s="2">
+        <f t="shared" si="1"/>
+        <v>164</v>
+      </c>
+      <c r="B186" t="s">
+        <v>33</v>
+      </c>
+      <c r="C186" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F186" s="13"/>
+      <c r="G186" s="13"/>
+      <c r="H186" s="11"/>
+      <c r="I186" s="11"/>
+    </row>
+    <row r="187" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A187" s="2">
+        <f t="shared" si="1"/>
+        <v>165</v>
+      </c>
+      <c r="B187" t="s">
+        <v>37</v>
+      </c>
+      <c r="C187" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F187" s="13"/>
+      <c r="G187" s="13"/>
+      <c r="H187" s="11"/>
+      <c r="I187" s="11"/>
+    </row>
+    <row r="188" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A188" s="2">
+        <f t="shared" si="1"/>
+        <v>166</v>
+      </c>
+      <c r="B188" t="s">
+        <v>37</v>
+      </c>
+      <c r="C188" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F188" s="13"/>
+      <c r="G188" s="13"/>
+      <c r="H188" s="11"/>
+      <c r="I188" s="11"/>
+    </row>
+    <row r="189" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A189" s="2">
+        <f t="shared" si="1"/>
+        <v>167</v>
+      </c>
+      <c r="B189" t="s">
+        <v>37</v>
+      </c>
+      <c r="C189" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F189" s="13"/>
+      <c r="G189" s="13"/>
+      <c r="H189" s="11"/>
+      <c r="I189" s="11"/>
+    </row>
+    <row r="190" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A190" s="2">
+        <f t="shared" si="1"/>
+        <v>168</v>
+      </c>
+      <c r="B190" t="s">
+        <v>38</v>
+      </c>
+      <c r="C190" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F190" s="13"/>
+      <c r="G190" s="13"/>
+      <c r="H190" s="11"/>
+      <c r="I190" s="11"/>
+    </row>
+    <row r="191" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A191" s="2">
+        <f t="shared" si="1"/>
+        <v>169</v>
+      </c>
+      <c r="B191" t="s">
+        <v>38</v>
+      </c>
+      <c r="C191" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F191" s="13"/>
+      <c r="G191" s="13"/>
+      <c r="H191" s="11"/>
+      <c r="I191" s="11"/>
+    </row>
+    <row r="192" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A192" s="2">
+        <f t="shared" si="1"/>
+        <v>170</v>
+      </c>
+      <c r="B192" t="s">
+        <v>38</v>
+      </c>
+      <c r="C192" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F192" s="13"/>
+      <c r="G192" s="13"/>
+      <c r="H192" s="11"/>
+      <c r="I192" s="11"/>
+    </row>
+    <row r="193" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A193" s="2">
+        <f t="shared" si="1"/>
+        <v>171</v>
+      </c>
+      <c r="B193" t="s">
+        <v>42</v>
+      </c>
+      <c r="C193" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F193" s="13"/>
+      <c r="G193" s="13"/>
+      <c r="H193" s="11"/>
+      <c r="I193" s="11"/>
+    </row>
+    <row r="194" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A194" s="2">
+        <f t="shared" ref="A194:A218" si="2">A193+1</f>
+        <v>172</v>
+      </c>
+      <c r="B194" t="s">
+        <v>42</v>
+      </c>
+      <c r="C194" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F194" s="13"/>
+      <c r="G194" s="13"/>
+      <c r="H194" s="11"/>
+      <c r="I194" s="11"/>
+    </row>
+    <row r="195" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A195" s="2">
+        <f t="shared" si="2"/>
+        <v>173</v>
+      </c>
+      <c r="B195" t="s">
+        <v>42</v>
+      </c>
+      <c r="C195" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F195" s="13"/>
+      <c r="G195" s="13"/>
+      <c r="H195" s="11"/>
+      <c r="I195" s="11"/>
+    </row>
+    <row r="196" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A196" s="2">
+        <f t="shared" si="2"/>
+        <v>174</v>
+      </c>
+      <c r="B196" t="s">
+        <v>46</v>
+      </c>
+      <c r="C196" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F196" s="13"/>
+      <c r="G196" s="13"/>
+      <c r="H196" s="11"/>
+      <c r="I196" s="11"/>
+    </row>
+    <row r="197" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A197" s="2">
+        <f t="shared" si="2"/>
+        <v>175</v>
+      </c>
+      <c r="B197" t="s">
+        <v>46</v>
+      </c>
+      <c r="C197" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F197" s="13"/>
+      <c r="G197" s="13"/>
+      <c r="H197" s="11"/>
+      <c r="I197" s="11"/>
+    </row>
+    <row r="198" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A198" s="2">
+        <f t="shared" si="2"/>
+        <v>176</v>
+      </c>
+      <c r="B198" t="s">
+        <v>46</v>
+      </c>
+      <c r="C198" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F198" s="13"/>
+      <c r="G198" s="13"/>
+      <c r="H198" s="11"/>
+      <c r="I198" s="11"/>
+    </row>
+    <row r="199" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A199" s="2">
+        <f t="shared" si="2"/>
+        <v>177</v>
+      </c>
+      <c r="B199" t="s">
+        <v>50</v>
+      </c>
+      <c r="C199" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F199" s="13"/>
+      <c r="G199" s="13"/>
+      <c r="H199" s="11"/>
+      <c r="I199" s="11"/>
+    </row>
+    <row r="200" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A200" s="2">
+        <f t="shared" si="2"/>
+        <v>178</v>
+      </c>
+      <c r="B200" t="s">
+        <v>50</v>
+      </c>
+      <c r="C200" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F200" s="13"/>
+      <c r="G200" s="13"/>
+      <c r="H200" s="11"/>
+      <c r="I200" s="11"/>
+    </row>
+    <row r="201" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A201" s="2">
+        <f t="shared" si="2"/>
+        <v>179</v>
+      </c>
+      <c r="B201" t="s">
+        <v>50</v>
+      </c>
+      <c r="C201" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F201" s="13"/>
+      <c r="G201" s="13"/>
+      <c r="H201" s="11"/>
+      <c r="I201" s="11"/>
+    </row>
+    <row r="202" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A202" s="2">
+        <f t="shared" si="2"/>
+        <v>180</v>
+      </c>
+      <c r="B202" t="s">
+        <v>51</v>
+      </c>
+      <c r="C202" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F202" s="13"/>
+      <c r="G202" s="13"/>
+      <c r="H202" s="11"/>
+      <c r="I202" s="11"/>
+    </row>
+    <row r="203" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A203" s="2">
+        <f t="shared" si="2"/>
+        <v>181</v>
+      </c>
+      <c r="B203" t="s">
+        <v>51</v>
+      </c>
+      <c r="C203" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F203" s="13"/>
+      <c r="G203" s="13"/>
+      <c r="H203" s="11"/>
+      <c r="I203" s="11"/>
+    </row>
+    <row r="204" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A204" s="2">
+        <f t="shared" si="2"/>
+        <v>182</v>
+      </c>
+      <c r="B204" t="s">
+        <v>51</v>
+      </c>
+      <c r="C204" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F204" s="13"/>
+      <c r="G204" s="13"/>
+      <c r="H204" s="11"/>
+      <c r="I204" s="11"/>
+    </row>
+    <row r="205" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A205" s="2">
+        <f t="shared" si="2"/>
+        <v>183</v>
+      </c>
+      <c r="B205" t="s">
+        <v>55</v>
+      </c>
+      <c r="C205" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F205" s="13"/>
+      <c r="G205" s="13"/>
+      <c r="H205" s="11"/>
+      <c r="I205" s="11"/>
+    </row>
+    <row r="206" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A206" s="2">
+        <f t="shared" si="2"/>
+        <v>184</v>
+      </c>
+      <c r="B206" t="s">
+        <v>55</v>
+      </c>
+      <c r="C206" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F206" s="13"/>
+      <c r="G206" s="13"/>
+      <c r="H206" s="11"/>
+      <c r="I206" s="11"/>
+    </row>
+    <row r="207" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A207" s="2">
+        <f t="shared" si="2"/>
+        <v>185</v>
+      </c>
+      <c r="B207" t="s">
+        <v>55</v>
+      </c>
+      <c r="C207" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F207" s="13"/>
+      <c r="G207" s="13"/>
+      <c r="H207" s="11"/>
+      <c r="I207" s="11"/>
+    </row>
+    <row r="208" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A208" s="2">
+        <f t="shared" si="2"/>
+        <v>186</v>
+      </c>
+      <c r="B208" t="s">
+        <v>59</v>
+      </c>
+      <c r="C208" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F208" s="13"/>
+      <c r="G208" s="13"/>
+      <c r="H208" s="11"/>
+      <c r="I208" s="11"/>
+    </row>
+    <row r="209" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A209" s="2">
+        <f t="shared" si="2"/>
+        <v>187</v>
+      </c>
+      <c r="B209" t="s">
+        <v>59</v>
+      </c>
+      <c r="C209" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F209" s="13"/>
+      <c r="G209" s="13"/>
+      <c r="H209" s="11"/>
+      <c r="I209" s="11"/>
+    </row>
+    <row r="210" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A210" s="2">
+        <f t="shared" si="2"/>
+        <v>188</v>
+      </c>
+      <c r="B210" t="s">
+        <v>59</v>
+      </c>
+      <c r="C210" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F210" s="13"/>
+      <c r="G210" s="13"/>
+      <c r="H210" s="11"/>
+      <c r="I210" s="11"/>
+    </row>
+    <row r="211" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A211" s="2">
+        <f t="shared" si="2"/>
+        <v>189</v>
+      </c>
+      <c r="B211" t="s">
+        <v>60</v>
+      </c>
+      <c r="C211" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F211" s="13"/>
+      <c r="G211" s="13"/>
+      <c r="H211" s="11"/>
+      <c r="I211" s="11"/>
+    </row>
+    <row r="212" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A212" s="2">
+        <f t="shared" si="2"/>
+        <v>190</v>
+      </c>
+      <c r="B212" t="s">
+        <v>60</v>
+      </c>
+      <c r="C212" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F212" s="13"/>
+      <c r="G212" s="13"/>
+      <c r="H212" s="11"/>
+      <c r="I212" s="11"/>
+    </row>
+    <row r="213" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A213" s="2">
+        <f t="shared" si="2"/>
+        <v>191</v>
+      </c>
+      <c r="B213" t="s">
+        <v>60</v>
+      </c>
+      <c r="C213" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F213" s="13"/>
+      <c r="G213" s="13"/>
+      <c r="H213" s="11"/>
+      <c r="I213" s="11"/>
+    </row>
+    <row r="214" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A214" s="2">
+        <f t="shared" si="2"/>
+        <v>192</v>
+      </c>
+      <c r="B214" t="s">
+        <v>63</v>
+      </c>
+      <c r="C214" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F214" s="13"/>
+      <c r="G214" s="13"/>
+      <c r="H214" s="11"/>
+      <c r="I214" s="11"/>
+    </row>
+    <row r="215" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A215" s="2">
+        <f t="shared" si="2"/>
+        <v>193</v>
+      </c>
+      <c r="B215" t="s">
+        <v>63</v>
+      </c>
+      <c r="C215" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="F215" s="13"/>
+      <c r="G215" s="13"/>
+      <c r="H215" s="11"/>
+      <c r="I215" s="11"/>
+    </row>
+    <row r="216" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A216" s="2">
+        <f t="shared" si="2"/>
+        <v>194</v>
+      </c>
+      <c r="B216" t="s">
+        <v>63</v>
+      </c>
+      <c r="C216" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F216" s="13"/>
+      <c r="G216" s="13"/>
+      <c r="H216" s="11"/>
+      <c r="I216" s="11"/>
+    </row>
+    <row r="217" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A217" s="2">
+        <f t="shared" si="2"/>
+        <v>195</v>
+      </c>
+      <c r="B217" t="s">
+        <v>67</v>
+      </c>
+      <c r="C217" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F217" s="13"/>
+      <c r="G217" s="13"/>
+      <c r="H217" s="11"/>
+      <c r="I217" s="11"/>
+    </row>
+    <row r="218" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A218" s="2">
+        <f t="shared" si="2"/>
+        <v>196</v>
+      </c>
+      <c r="B218" t="s">
+        <v>67</v>
+      </c>
+      <c r="C218" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="F218" s="13"/>
+      <c r="G218" s="13"/>
+      <c r="H218" s="11"/>
+      <c r="I218" s="11"/>
+    </row>
+    <row r="219" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A219" s="2">
+        <f t="shared" ref="A219" si="3">A218+1</f>
+        <v>197</v>
+      </c>
+      <c r="B219" t="s">
+        <v>67</v>
+      </c>
+      <c r="C219" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F219" s="13"/>
+      <c r="G219" s="13"/>
+      <c r="H219" s="11"/>
+      <c r="I219" s="11"/>
+    </row>
+    <row r="220" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="221" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="222" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="223" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="224" spans="1:9" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="225" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="226" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="227" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="228" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="229" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="230" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="231" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="232" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="233" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="234" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="235" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="236" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="237" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="238" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="239" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="240" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="241" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="242" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="243" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="244" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="245" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="246" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="247" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="248" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="249" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="250" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="251" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="252" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="253" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="254" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="255" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="256" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="257" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="258" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="259" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="260" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="261" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="262" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="263" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="264" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="265" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="266" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="267" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="268" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="269" ht="20.350000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>
-  <autoFilter ref="A1:I157" xr:uid="{53B5725F-EA7B-4922-8CC3-F684A90DDE36}"/>
-  <conditionalFormatting sqref="D2:D13 D15:D16 D18:D19 D21:D70 D72:D157">
+  <autoFilter ref="A1:I219" xr:uid="{53B5725F-EA7B-4922-8CC3-F684A90DDE36}"/>
+  <conditionalFormatting sqref="D2:D13 D15:D16 D18:D19 D21:D70 D72:D219">
     <cfRule type="cellIs" dxfId="9" priority="9" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -4912,11 +6034,129 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D169" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D231" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Pass,Fail"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74EA7C95-069C-40BA-B0DC-A7B8FEEBE296}">
+  <dimension ref="B4:B5"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="4" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B4" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B5" t="s">
+        <v>251</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20554CEA-9385-4992-8E38-F6F506B6C8CB}">
+  <dimension ref="C7:C23"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="7" spans="3:3" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="C7" s="8" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="8" spans="3:3" x14ac:dyDescent="0.45">
+      <c r="C8" s="8" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="9" spans="3:3" x14ac:dyDescent="0.45">
+      <c r="C9" s="8" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="10" spans="3:3" x14ac:dyDescent="0.45">
+      <c r="C10" s="8" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="11" spans="3:3" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="C11" s="8" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="12" spans="3:3" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="C12" s="8" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="13" spans="3:3" x14ac:dyDescent="0.45">
+      <c r="C13" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="3:3" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="C14" s="8" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="15" spans="3:3" x14ac:dyDescent="0.45">
+      <c r="C15" s="8" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="16" spans="3:3" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="C16" s="8" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="17" spans="3:3" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="C17" s="8" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="18" spans="3:3" x14ac:dyDescent="0.45">
+      <c r="C18" s="8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" spans="3:3" x14ac:dyDescent="0.45">
+      <c r="C19" s="8" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="20" spans="3:3" x14ac:dyDescent="0.45">
+      <c r="C20" s="8" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="21" spans="3:3" x14ac:dyDescent="0.45">
+      <c r="C21" s="8" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="22" spans="3:3" x14ac:dyDescent="0.45">
+      <c r="C22" s="8" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="23" spans="3:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="C23" s="6" t="s">
+        <v>215</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState ref="C7:C23">
+    <sortCondition ref="C7:C23"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>